<commit_message>
Add 6 spare rows to SEL biennial analogue measurements section
Generator relays (SEL-300G, SEL-700G) have additional current inputs
(Y-side 87 CTs, neutral, differential quantities) beyond the 8 standard
rows. Spare rows left blank for technician to fill in quantity/unit.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SEL_Biennial_Visual_Check.xlsx
+++ b/SEL_Biennial_Visual_Check.xlsx
@@ -185,7 +185,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -217,14 +217,23 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -637,7 +646,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E90"/>
+  <dimension ref="A1:E96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -660,10 +669,10 @@
           <t>1.  RELAY AND SITE INFORMATION</t>
         </is>
       </c>
-      <c r="B3" s="17" t="n"/>
-      <c r="C3" s="17" t="n"/>
-      <c r="D3" s="17" t="n"/>
-      <c r="E3" s="18" t="n"/>
+      <c r="B3" s="20" t="n"/>
+      <c r="C3" s="20" t="n"/>
+      <c r="D3" s="20" t="n"/>
+      <c r="E3" s="21" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -676,9 +685,9 @@
           <t>SEL-300G  /  SEL-311L  /  SEL-787  /  SEL-700G  (circle one)</t>
         </is>
       </c>
-      <c r="C4" s="17" t="n"/>
-      <c r="D4" s="17" t="n"/>
-      <c r="E4" s="18" t="n"/>
+      <c r="C4" s="20" t="n"/>
+      <c r="D4" s="20" t="n"/>
+      <c r="E4" s="21" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -687,9 +696,9 @@
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr"/>
-      <c r="C5" s="17" t="n"/>
-      <c r="D5" s="17" t="n"/>
-      <c r="E5" s="18" t="n"/>
+      <c r="C5" s="20" t="n"/>
+      <c r="D5" s="20" t="n"/>
+      <c r="E5" s="21" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -698,9 +707,9 @@
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr"/>
-      <c r="C6" s="17" t="n"/>
-      <c r="D6" s="17" t="n"/>
-      <c r="E6" s="18" t="n"/>
+      <c r="C6" s="20" t="n"/>
+      <c r="D6" s="20" t="n"/>
+      <c r="E6" s="21" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -709,9 +718,9 @@
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr"/>
-      <c r="C7" s="17" t="n"/>
-      <c r="D7" s="17" t="n"/>
-      <c r="E7" s="18" t="n"/>
+      <c r="C7" s="20" t="n"/>
+      <c r="D7" s="20" t="n"/>
+      <c r="E7" s="21" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -720,9 +729,9 @@
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr"/>
-      <c r="C8" s="17" t="n"/>
-      <c r="D8" s="17" t="n"/>
-      <c r="E8" s="18" t="n"/>
+      <c r="C8" s="20" t="n"/>
+      <c r="D8" s="20" t="n"/>
+      <c r="E8" s="21" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -731,9 +740,9 @@
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr"/>
-      <c r="C9" s="17" t="n"/>
-      <c r="D9" s="17" t="n"/>
-      <c r="E9" s="18" t="n"/>
+      <c r="C9" s="20" t="n"/>
+      <c r="D9" s="20" t="n"/>
+      <c r="E9" s="21" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -742,9 +751,9 @@
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr"/>
-      <c r="C10" s="17" t="n"/>
-      <c r="D10" s="17" t="n"/>
-      <c r="E10" s="18" t="n"/>
+      <c r="C10" s="20" t="n"/>
+      <c r="D10" s="20" t="n"/>
+      <c r="E10" s="21" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -753,9 +762,9 @@
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr"/>
-      <c r="C11" s="17" t="n"/>
-      <c r="D11" s="17" t="n"/>
-      <c r="E11" s="18" t="n"/>
+      <c r="C11" s="20" t="n"/>
+      <c r="D11" s="20" t="n"/>
+      <c r="E11" s="21" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -768,9 +777,9 @@
           <t>(2 years from date above)</t>
         </is>
       </c>
-      <c r="C12" s="17" t="n"/>
-      <c r="D12" s="17" t="n"/>
-      <c r="E12" s="18" t="n"/>
+      <c r="C12" s="20" t="n"/>
+      <c r="D12" s="20" t="n"/>
+      <c r="E12" s="21" t="n"/>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
@@ -778,10 +787,10 @@
           <t>2.  CONNECTION METHOD</t>
         </is>
       </c>
-      <c r="B14" s="17" t="n"/>
-      <c r="C14" s="17" t="n"/>
-      <c r="D14" s="17" t="n"/>
-      <c r="E14" s="18" t="n"/>
+      <c r="B14" s="20" t="n"/>
+      <c r="C14" s="20" t="n"/>
+      <c r="D14" s="20" t="n"/>
+      <c r="E14" s="21" t="n"/>
     </row>
     <row r="15" ht="52" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
@@ -791,10 +800,10 @@
 OPTION C — Ethernet (if fitted): Open AcSELerator QuickSet or SSH/Telnet to relay IP.</t>
         </is>
       </c>
-      <c r="B15" s="17" t="n"/>
-      <c r="C15" s="17" t="n"/>
-      <c r="D15" s="17" t="n"/>
-      <c r="E15" s="18" t="n"/>
+      <c r="B15" s="20" t="n"/>
+      <c r="C15" s="20" t="n"/>
+      <c r="D15" s="20" t="n"/>
+      <c r="E15" s="21" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -807,9 +816,9 @@
           <t>Front panel / Serial cable / Ethernet  (delete as applicable)</t>
         </is>
       </c>
-      <c r="C16" s="17" t="n"/>
-      <c r="D16" s="17" t="n"/>
-      <c r="E16" s="18" t="n"/>
+      <c r="C16" s="20" t="n"/>
+      <c r="D16" s="20" t="n"/>
+      <c r="E16" s="21" t="n"/>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
@@ -817,10 +826,10 @@
           <t>3.  SELF-TEST AND DEVICE STATUS</t>
         </is>
       </c>
-      <c r="B18" s="17" t="n"/>
-      <c r="C18" s="17" t="n"/>
-      <c r="D18" s="17" t="n"/>
-      <c r="E18" s="18" t="n"/>
+      <c r="B18" s="20" t="n"/>
+      <c r="C18" s="20" t="n"/>
+      <c r="D18" s="20" t="n"/>
+      <c r="E18" s="21" t="n"/>
     </row>
     <row r="19" ht="36" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
@@ -828,10 +837,10 @@
           <t>Front panel: ENABLED LED (green, solid) must be illuminated. Serial: type STA &lt;Enter&gt; or STATUS &lt;Enter&gt; — all items should show OK. W = warning (issue STA C to clear), FAIL = fault (requires investigation).</t>
         </is>
       </c>
-      <c r="B19" s="17" t="n"/>
-      <c r="C19" s="17" t="n"/>
-      <c r="D19" s="17" t="n"/>
-      <c r="E19" s="18" t="n"/>
+      <c r="B19" s="20" t="n"/>
+      <c r="C19" s="20" t="n"/>
+      <c r="D19" s="20" t="n"/>
+      <c r="E19" s="21" t="n"/>
     </row>
     <row r="20" ht="28" customHeight="1">
       <c r="A20" s="6" t="inlineStr">
@@ -1000,10 +1009,10 @@
           <t>4.  ANALOGUE MEASUREMENTS  (Primary Values — relay reports in primary units)</t>
         </is>
       </c>
-      <c r="B29" s="17" t="n"/>
-      <c r="C29" s="17" t="n"/>
-      <c r="D29" s="17" t="n"/>
-      <c r="E29" s="18" t="n"/>
+      <c r="B29" s="20" t="n"/>
+      <c r="C29" s="20" t="n"/>
+      <c r="D29" s="20" t="n"/>
+      <c r="E29" s="21" t="n"/>
     </row>
     <row r="30" ht="40" customHeight="1">
       <c r="A30" s="5" t="inlineStr">
@@ -1011,10 +1020,10 @@
           <t>Serial: type METER &lt;Enter&gt; — relay displays primary values (A and V). Front panel: Main &gt; Meters &gt; Fundamental.  Record measured values. Compare to expected load (no specific pass/fail for 2-yearly — flag anything obviously wrong, e.g., one phase zero when others are normal).</t>
         </is>
       </c>
-      <c r="B30" s="17" t="n"/>
-      <c r="C30" s="17" t="n"/>
-      <c r="D30" s="17" t="n"/>
-      <c r="E30" s="18" t="n"/>
+      <c r="B30" s="20" t="n"/>
+      <c r="C30" s="20" t="n"/>
+      <c r="D30" s="20" t="n"/>
+      <c r="E30" s="21" t="n"/>
     </row>
     <row r="31" ht="28" customHeight="1">
       <c r="A31" s="6" t="inlineStr">
@@ -1198,631 +1207,697 @@
       </c>
       <c r="E39" s="4" t="n"/>
     </row>
-    <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="2" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="11" t="inlineStr"/>
+      <c r="B40" s="9" t="inlineStr">
+        <is>
+          <t>METER / Meters &gt; Fundamental</t>
+        </is>
+      </c>
+      <c r="C40" s="12" t="n"/>
+      <c r="D40" s="13" t="n"/>
+      <c r="E40" s="13" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="14" t="inlineStr"/>
+      <c r="B41" s="9" t="inlineStr">
+        <is>
+          <t>METER / Meters &gt; Fundamental</t>
+        </is>
+      </c>
+      <c r="C41" s="10" t="n"/>
+      <c r="D41" s="4" t="n"/>
+      <c r="E41" s="4" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="11" t="inlineStr"/>
+      <c r="B42" s="9" t="inlineStr">
+        <is>
+          <t>METER / Meters &gt; Fundamental</t>
+        </is>
+      </c>
+      <c r="C42" s="12" t="n"/>
+      <c r="D42" s="13" t="n"/>
+      <c r="E42" s="13" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="14" t="inlineStr"/>
+      <c r="B43" s="9" t="inlineStr">
+        <is>
+          <t>METER / Meters &gt; Fundamental</t>
+        </is>
+      </c>
+      <c r="C43" s="10" t="n"/>
+      <c r="D43" s="4" t="n"/>
+      <c r="E43" s="4" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="11" t="inlineStr"/>
+      <c r="B44" s="9" t="inlineStr">
+        <is>
+          <t>METER / Meters &gt; Fundamental</t>
+        </is>
+      </c>
+      <c r="C44" s="12" t="n"/>
+      <c r="D44" s="13" t="n"/>
+      <c r="E44" s="13" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="14" t="inlineStr"/>
+      <c r="B45" s="9" t="inlineStr">
+        <is>
+          <t>METER / Meters &gt; Fundamental</t>
+        </is>
+      </c>
+      <c r="C45" s="10" t="n"/>
+      <c r="D45" s="4" t="n"/>
+      <c r="E45" s="4" t="n"/>
+    </row>
+    <row r="47" ht="18" customHeight="1">
+      <c r="A47" s="2" t="inlineStr">
         <is>
           <t>5.  CLOCK AND TIME SYNCHRONISATION</t>
         </is>
       </c>
-      <c r="B41" s="17" t="n"/>
-      <c r="C41" s="17" t="n"/>
-      <c r="D41" s="17" t="n"/>
-      <c r="E41" s="18" t="n"/>
-    </row>
-    <row r="42" ht="28" customHeight="1">
-      <c r="A42" s="6" t="inlineStr">
+      <c r="B47" s="20" t="n"/>
+      <c r="C47" s="20" t="n"/>
+      <c r="D47" s="20" t="n"/>
+      <c r="E47" s="21" t="n"/>
+    </row>
+    <row r="48" ht="28" customHeight="1">
+      <c r="A48" s="6" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
       </c>
-      <c r="B42" s="6" t="inlineStr">
+      <c r="B48" s="6" t="inlineStr">
         <is>
           <t>How to Read</t>
         </is>
       </c>
-      <c r="C42" s="6" t="inlineStr">
+      <c r="C48" s="6" t="inlineStr">
         <is>
           <t>Relay Value</t>
         </is>
       </c>
-      <c r="D42" s="6" t="inlineStr">
+      <c r="D48" s="6" t="inlineStr">
         <is>
           <t>Reference Value</t>
         </is>
       </c>
-      <c r="E42" s="6" t="inlineStr">
+      <c r="E48" s="6" t="inlineStr">
         <is>
           <t>Difference / Result</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="7" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="7" t="inlineStr">
         <is>
           <t>Relay Date</t>
         </is>
       </c>
-      <c r="B43" s="8" t="inlineStr">
+      <c r="B49" s="8" t="inlineStr">
         <is>
           <t>Serial: DAT &lt;Enter&gt;
 Front panel: Main &gt; Time or Status</t>
         </is>
       </c>
-      <c r="C43" s="10" t="inlineStr"/>
-      <c r="D43" s="9" t="inlineStr">
+      <c r="C49" s="10" t="inlineStr"/>
+      <c r="D49" s="9" t="inlineStr">
         <is>
           <t>Today's date</t>
         </is>
       </c>
-      <c r="E43" s="4" t="n"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="7" t="inlineStr">
+      <c r="E49" s="4" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="7" t="inlineStr">
         <is>
           <t>Relay Time</t>
         </is>
       </c>
-      <c r="B44" s="8" t="inlineStr">
+      <c r="B50" s="8" t="inlineStr">
         <is>
           <t>Serial: TIM &lt;Enter&gt;
 Front panel: Main &gt; Time or Status</t>
         </is>
       </c>
-      <c r="C44" s="10" t="inlineStr"/>
-      <c r="D44" s="9" t="inlineStr">
+      <c r="C50" s="10" t="inlineStr"/>
+      <c r="D50" s="9" t="inlineStr">
         <is>
           <t>GPS/NTP reference</t>
         </is>
       </c>
-      <c r="E44" s="4" t="n"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="7" t="inlineStr">
+      <c r="E50" s="4" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="7" t="inlineStr">
         <is>
           <t>Time source (IRIG-B / NTP / Internal)</t>
         </is>
       </c>
-      <c r="B45" s="8" t="inlineStr">
+      <c r="B51" s="8" t="inlineStr">
         <is>
           <t>Serial: STA &lt;Enter&gt; — look for IRIG-B or NTP line</t>
         </is>
       </c>
-      <c r="C45" s="10" t="inlineStr"/>
-      <c r="D45" s="9" t="inlineStr">
+      <c r="C51" s="10" t="inlineStr"/>
+      <c r="D51" s="9" t="inlineStr">
         <is>
           <t>IRIG-B preferred</t>
         </is>
       </c>
-      <c r="E45" s="4" t="n"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="7" t="inlineStr">
+      <c r="E51" s="4" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="7" t="inlineStr">
         <is>
           <t>Time difference (accept ≤ 10 s)</t>
         </is>
       </c>
-      <c r="B46" s="8" t="inlineStr">
+      <c r="B52" s="8" t="inlineStr">
         <is>
           <t>Relay time vs phone/GPS reference</t>
         </is>
       </c>
-      <c r="C46" s="10" t="inlineStr"/>
-      <c r="D46" s="9" t="inlineStr">
+      <c r="C52" s="10" t="inlineStr"/>
+      <c r="D52" s="9" t="inlineStr">
         <is>
           <t>≤ 10 s</t>
         </is>
       </c>
-      <c r="E46" s="4" t="n"/>
-    </row>
-    <row r="48" ht="18" customHeight="1">
-      <c r="A48" s="2" t="inlineStr">
+      <c r="E52" s="4" t="n"/>
+    </row>
+    <row r="54" ht="18" customHeight="1">
+      <c r="A54" s="2" t="inlineStr">
         <is>
           <t>6.  RECENT EVENTS  (record most recent events — flag any unexplained trips or alarms)</t>
         </is>
       </c>
-      <c r="B48" s="17" t="n"/>
-      <c r="C48" s="17" t="n"/>
-      <c r="D48" s="17" t="n"/>
-      <c r="E48" s="18" t="n"/>
-    </row>
-    <row r="49" ht="36" customHeight="1">
-      <c r="A49" s="5" t="inlineStr">
+      <c r="B54" s="20" t="n"/>
+      <c r="C54" s="20" t="n"/>
+      <c r="D54" s="20" t="n"/>
+      <c r="E54" s="21" t="n"/>
+    </row>
+    <row r="55" ht="36" customHeight="1">
+      <c r="A55" s="5" t="inlineStr">
         <is>
           <t>Serial: type HIS &lt;Enter&gt; for event history, or EVE &lt;Enter&gt; for last event report, or SER &lt;Enter&gt; for Sequential Events Recorder.  Front panel: Main &gt; Events (or Main &gt; Targets for relay word bits).  Record the most recent events and their dates below.</t>
         </is>
       </c>
-      <c r="B49" s="17" t="n"/>
-      <c r="C49" s="17" t="n"/>
-      <c r="D49" s="17" t="n"/>
-      <c r="E49" s="18" t="n"/>
-    </row>
-    <row r="50" ht="28" customHeight="1">
-      <c r="A50" s="6" t="inlineStr">
+      <c r="B55" s="20" t="n"/>
+      <c r="C55" s="20" t="n"/>
+      <c r="D55" s="20" t="n"/>
+      <c r="E55" s="21" t="n"/>
+    </row>
+    <row r="56" ht="28" customHeight="1">
+      <c r="A56" s="6" t="inlineStr">
         <is>
           <t>Event #
 (most recent = 1)</t>
         </is>
       </c>
-      <c r="B50" s="6" t="inlineStr">
+      <c r="B56" s="6" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="C50" s="6" t="inlineStr">
+      <c r="C56" s="6" t="inlineStr">
         <is>
           <t>Time</t>
         </is>
       </c>
-      <c r="D50" s="6" t="inlineStr">
+      <c r="D56" s="6" t="inlineStr">
         <is>
           <t>Event Description / Type</t>
         </is>
       </c>
-      <c r="E50" s="18" t="n"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="11" t="n">
+      <c r="E56" s="21" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="15" t="n">
         <v>1</v>
-      </c>
-      <c r="B51" s="4" t="n"/>
-      <c r="C51" s="4" t="n"/>
-      <c r="D51" s="4" t="n"/>
-      <c r="E51" s="18" t="n"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="B52" s="13" t="n"/>
-      <c r="C52" s="13" t="n"/>
-      <c r="D52" s="13" t="n"/>
-      <c r="E52" s="18" t="n"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="B53" s="4" t="n"/>
-      <c r="C53" s="4" t="n"/>
-      <c r="D53" s="4" t="n"/>
-      <c r="E53" s="18" t="n"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="B54" s="13" t="n"/>
-      <c r="C54" s="13" t="n"/>
-      <c r="D54" s="13" t="n"/>
-      <c r="E54" s="18" t="n"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="11" t="n">
-        <v>5</v>
-      </c>
-      <c r="B55" s="4" t="n"/>
-      <c r="C55" s="4" t="n"/>
-      <c r="D55" s="4" t="n"/>
-      <c r="E55" s="18" t="n"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="12" t="n">
-        <v>6</v>
-      </c>
-      <c r="B56" s="13" t="n"/>
-      <c r="C56" s="13" t="n"/>
-      <c r="D56" s="13" t="n"/>
-      <c r="E56" s="18" t="n"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="11" t="n">
-        <v>7</v>
       </c>
       <c r="B57" s="4" t="n"/>
       <c r="C57" s="4" t="n"/>
       <c r="D57" s="4" t="n"/>
-      <c r="E57" s="18" t="n"/>
+      <c r="E57" s="21" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="12" t="n">
-        <v>8</v>
+      <c r="A58" s="16" t="n">
+        <v>2</v>
       </c>
       <c r="B58" s="13" t="n"/>
       <c r="C58" s="13" t="n"/>
       <c r="D58" s="13" t="n"/>
-      <c r="E58" s="18" t="n"/>
+      <c r="E58" s="21" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="11" t="n">
-        <v>9</v>
+      <c r="A59" s="15" t="n">
+        <v>3</v>
       </c>
       <c r="B59" s="4" t="n"/>
       <c r="C59" s="4" t="n"/>
       <c r="D59" s="4" t="n"/>
-      <c r="E59" s="18" t="n"/>
+      <c r="E59" s="21" t="n"/>
     </row>
     <row r="60">
-      <c r="A60" s="12" t="n">
-        <v>10</v>
+      <c r="A60" s="16" t="n">
+        <v>4</v>
       </c>
       <c r="B60" s="13" t="n"/>
       <c r="C60" s="13" t="n"/>
       <c r="D60" s="13" t="n"/>
-      <c r="E60" s="18" t="n"/>
+      <c r="E60" s="21" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" s="11" t="n">
-        <v>11</v>
+      <c r="A61" s="15" t="n">
+        <v>5</v>
       </c>
       <c r="B61" s="4" t="n"/>
       <c r="C61" s="4" t="n"/>
       <c r="D61" s="4" t="n"/>
-      <c r="E61" s="18" t="n"/>
+      <c r="E61" s="21" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="12" t="n">
-        <v>12</v>
+      <c r="A62" s="16" t="n">
+        <v>6</v>
       </c>
       <c r="B62" s="13" t="n"/>
       <c r="C62" s="13" t="n"/>
       <c r="D62" s="13" t="n"/>
-      <c r="E62" s="18" t="n"/>
+      <c r="E62" s="21" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" s="3" t="inlineStr">
+      <c r="A63" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="B63" s="4" t="n"/>
+      <c r="C63" s="4" t="n"/>
+      <c r="D63" s="4" t="n"/>
+      <c r="E63" s="21" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="16" t="n">
+        <v>8</v>
+      </c>
+      <c r="B64" s="13" t="n"/>
+      <c r="C64" s="13" t="n"/>
+      <c r="D64" s="13" t="n"/>
+      <c r="E64" s="21" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="B65" s="4" t="n"/>
+      <c r="C65" s="4" t="n"/>
+      <c r="D65" s="4" t="n"/>
+      <c r="E65" s="21" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="B66" s="13" t="n"/>
+      <c r="C66" s="13" t="n"/>
+      <c r="D66" s="13" t="n"/>
+      <c r="E66" s="21" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="15" t="n">
+        <v>11</v>
+      </c>
+      <c r="B67" s="4" t="n"/>
+      <c r="C67" s="4" t="n"/>
+      <c r="D67" s="4" t="n"/>
+      <c r="E67" s="21" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="16" t="n">
+        <v>12</v>
+      </c>
+      <c r="B68" s="13" t="n"/>
+      <c r="C68" s="13" t="n"/>
+      <c r="D68" s="13" t="n"/>
+      <c r="E68" s="21" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="3" t="inlineStr">
         <is>
           <t>Total events since last check (approx.)</t>
         </is>
       </c>
-      <c r="B63" s="4" t="n"/>
-      <c r="C63" s="17" t="n"/>
-      <c r="D63" s="17" t="n"/>
-      <c r="E63" s="18" t="n"/>
-    </row>
-    <row r="65" ht="18" customHeight="1">
-      <c r="A65" s="2" t="inlineStr">
+      <c r="B69" s="4" t="n"/>
+      <c r="C69" s="20" t="n"/>
+      <c r="D69" s="20" t="n"/>
+      <c r="E69" s="21" t="n"/>
+    </row>
+    <row r="71" ht="18" customHeight="1">
+      <c r="A71" s="2" t="inlineStr">
         <is>
           <t>7.  DCS / 800XA COMMUNICATION CHECK</t>
         </is>
       </c>
-      <c r="B65" s="17" t="n"/>
-      <c r="C65" s="17" t="n"/>
-      <c r="D65" s="17" t="n"/>
-      <c r="E65" s="18" t="n"/>
-    </row>
-    <row r="66" ht="36" customHeight="1">
-      <c r="A66" s="5" t="inlineStr">
+      <c r="B71" s="20" t="n"/>
+      <c r="C71" s="20" t="n"/>
+      <c r="D71" s="20" t="n"/>
+      <c r="E71" s="21" t="n"/>
+    </row>
+    <row r="72" ht="36" customHeight="1">
+      <c r="A72" s="5" t="inlineStr">
         <is>
           <t>Open the relay faceplate in ABB 800XA. Verify that live values (currents, status) are updating and not frozen. Check for any communication alarm objects (yellow/red). Record the 800XA object path or faceplate name below.</t>
         </is>
       </c>
-      <c r="B66" s="17" t="n"/>
-      <c r="C66" s="17" t="n"/>
-      <c r="D66" s="17" t="n"/>
-      <c r="E66" s="18" t="n"/>
-    </row>
-    <row r="67" ht="28" customHeight="1">
-      <c r="A67" s="6" t="inlineStr">
+      <c r="B72" s="20" t="n"/>
+      <c r="C72" s="20" t="n"/>
+      <c r="D72" s="20" t="n"/>
+      <c r="E72" s="21" t="n"/>
+    </row>
+    <row r="73" ht="28" customHeight="1">
+      <c r="A73" s="6" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
       </c>
-      <c r="B67" s="6" t="inlineStr">
+      <c r="B73" s="6" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="C67" s="6" t="inlineStr">
+      <c r="C73" s="6" t="inlineStr">
         <is>
           <t>Result
 (Y / N)</t>
         </is>
       </c>
-      <c r="D67" s="6" t="inlineStr">
+      <c r="D73" s="6" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="E67" s="18" t="n"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="3" t="inlineStr">
+      <c r="E73" s="21" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="3" t="inlineStr">
         <is>
           <t>800XA faceplate opened</t>
         </is>
       </c>
-      <c r="B68" s="9" t="inlineStr">
+      <c r="B74" s="9" t="inlineStr">
         <is>
           <t>Navigate to relay faceplate in 800XA control system</t>
         </is>
       </c>
-      <c r="C68" s="10" t="n"/>
-      <c r="D68" s="4" t="n"/>
-      <c r="E68" s="18" t="n"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="3" t="inlineStr">
+      <c r="C74" s="10" t="n"/>
+      <c r="D74" s="4" t="n"/>
+      <c r="E74" s="21" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="3" t="inlineStr">
         <is>
           <t>Live values updating</t>
         </is>
       </c>
-      <c r="B69" s="9" t="inlineStr">
+      <c r="B75" s="9" t="inlineStr">
         <is>
           <t>Phase currents / status visible and changing with load — not frozen</t>
         </is>
       </c>
-      <c r="C69" s="10" t="n"/>
-      <c r="D69" s="4" t="n"/>
-      <c r="E69" s="18" t="n"/>
-    </row>
-    <row r="70">
-      <c r="A70" s="3" t="inlineStr">
+      <c r="C75" s="10" t="n"/>
+      <c r="D75" s="4" t="n"/>
+      <c r="E75" s="21" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="3" t="inlineStr">
         <is>
           <t>No communication alarm</t>
         </is>
       </c>
-      <c r="B70" s="9" t="inlineStr">
+      <c r="B76" s="9" t="inlineStr">
         <is>
           <t>No yellow or red communication alarm objects on faceplate</t>
         </is>
       </c>
-      <c r="C70" s="10" t="n"/>
-      <c r="D70" s="4" t="n"/>
-      <c r="E70" s="18" t="n"/>
-    </row>
-    <row r="71">
-      <c r="A71" s="3" t="inlineStr">
+      <c r="C76" s="10" t="n"/>
+      <c r="D76" s="4" t="n"/>
+      <c r="E76" s="21" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="3" t="inlineStr">
         <is>
           <t>Record 800XA object path / faceplate name</t>
         </is>
       </c>
-      <c r="B71" s="9" t="inlineStr">
+      <c r="B77" s="9" t="inlineStr">
         <is>
           <t>e.g. "Site/Substation/Relay Tag/Faceplate"</t>
         </is>
       </c>
-      <c r="C71" s="10" t="n"/>
-      <c r="D71" s="4" t="n"/>
-      <c r="E71" s="18" t="n"/>
-    </row>
-    <row r="73" ht="18" customHeight="1">
-      <c r="A73" s="2" t="inlineStr">
+      <c r="C77" s="10" t="n"/>
+      <c r="D77" s="4" t="n"/>
+      <c r="E77" s="21" t="n"/>
+    </row>
+    <row r="79" ht="18" customHeight="1">
+      <c r="A79" s="2" t="inlineStr">
         <is>
           <t>8.  OPTIONAL — CLEAR EVENT BUFFERS  (only if required by your procedure)</t>
         </is>
       </c>
-      <c r="B73" s="17" t="n"/>
-      <c r="C73" s="17" t="n"/>
-      <c r="D73" s="17" t="n"/>
-      <c r="E73" s="18" t="n"/>
-    </row>
-    <row r="74" ht="32" customHeight="1">
-      <c r="A74" s="14" t="inlineStr">
+      <c r="B79" s="20" t="n"/>
+      <c r="C79" s="20" t="n"/>
+      <c r="D79" s="20" t="n"/>
+      <c r="E79" s="21" t="n"/>
+    </row>
+    <row r="80" ht="32" customHeight="1">
+      <c r="A80" s="17" t="inlineStr">
         <is>
           <t>If your site procedure requires clearing event buffers after recording, issue the following serial commands at Access Level 1 or 2. Ensure all events have been downloaded/recorded BEFORE clearing.</t>
         </is>
       </c>
-      <c r="B74" s="17" t="n"/>
-      <c r="C74" s="17" t="n"/>
-      <c r="D74" s="17" t="n"/>
-      <c r="E74" s="18" t="n"/>
-    </row>
-    <row r="75" ht="28" customHeight="1">
-      <c r="A75" s="6" t="inlineStr">
+      <c r="B80" s="20" t="n"/>
+      <c r="C80" s="20" t="n"/>
+      <c r="D80" s="20" t="n"/>
+      <c r="E80" s="21" t="n"/>
+    </row>
+    <row r="81" ht="28" customHeight="1">
+      <c r="A81" s="6" t="inlineStr">
         <is>
           <t>Serial Command</t>
         </is>
       </c>
-      <c r="B75" s="6" t="inlineStr">
+      <c r="B81" s="6" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="C75" s="6" t="inlineStr">
+      <c r="C81" s="6" t="inlineStr">
         <is>
           <t>Performed?
 (Y / N / N/A)</t>
         </is>
       </c>
-      <c r="D75" s="6" t="inlineStr">
+      <c r="D81" s="6" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="E75" s="18" t="n"/>
-    </row>
-    <row r="76">
-      <c r="A76" s="3" t="inlineStr">
+      <c r="E81" s="21" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="3" t="inlineStr">
         <is>
           <t>SUM R &lt;Enter&gt;</t>
         </is>
       </c>
-      <c r="B76" s="9" t="inlineStr">
+      <c r="B82" s="9" t="inlineStr">
         <is>
           <t>Reset event report and Summary Command buffers</t>
         </is>
       </c>
-      <c r="C76" s="10" t="n"/>
-      <c r="D76" s="4" t="n"/>
-      <c r="E76" s="18" t="n"/>
-    </row>
-    <row r="77">
-      <c r="A77" s="3" t="inlineStr">
+      <c r="C82" s="10" t="n"/>
+      <c r="D82" s="4" t="n"/>
+      <c r="E82" s="21" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="3" t="inlineStr">
         <is>
           <t>SER R &lt;Enter&gt;</t>
         </is>
       </c>
-      <c r="B77" s="9" t="inlineStr">
+      <c r="B83" s="9" t="inlineStr">
         <is>
           <t>Reset Sequential Events Record buffer</t>
         </is>
       </c>
-      <c r="C77" s="10" t="n"/>
-      <c r="D77" s="4" t="n"/>
-      <c r="E77" s="18" t="n"/>
-    </row>
-    <row r="78">
-      <c r="A78" s="3" t="inlineStr">
+      <c r="C83" s="10" t="n"/>
+      <c r="D83" s="4" t="n"/>
+      <c r="E83" s="21" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="3" t="inlineStr">
         <is>
           <t>HIS C &lt;Enter&gt;</t>
         </is>
       </c>
-      <c r="B78" s="9" t="inlineStr">
+      <c r="B84" s="9" t="inlineStr">
         <is>
           <t>Clear event history (if required — confirm with supervisor)</t>
         </is>
       </c>
-      <c r="C78" s="10" t="n"/>
-      <c r="D78" s="4" t="n"/>
-      <c r="E78" s="18" t="n"/>
-    </row>
-    <row r="80" ht="18" customHeight="1">
-      <c r="A80" s="2" t="inlineStr">
+      <c r="C84" s="10" t="n"/>
+      <c r="D84" s="4" t="n"/>
+      <c r="E84" s="21" t="n"/>
+    </row>
+    <row r="86" ht="18" customHeight="1">
+      <c r="A86" s="2" t="inlineStr">
         <is>
           <t>9.  OBSERVATIONS AND CORRECTIVE ACTIONS</t>
         </is>
       </c>
-      <c r="B80" s="17" t="n"/>
-      <c r="C80" s="17" t="n"/>
-      <c r="D80" s="17" t="n"/>
-      <c r="E80" s="18" t="n"/>
-    </row>
-    <row r="81" ht="18" customHeight="1">
-      <c r="A81" s="15" t="n"/>
-      <c r="B81" s="19" t="n"/>
-      <c r="C81" s="19" t="n"/>
-      <c r="D81" s="19" t="n"/>
-      <c r="E81" s="20" t="n"/>
-    </row>
-    <row r="82" ht="18" customHeight="1">
-      <c r="A82" s="21" t="n"/>
-      <c r="E82" s="22" t="n"/>
-    </row>
-    <row r="83" ht="18" customHeight="1">
-      <c r="A83" s="21" t="n"/>
-      <c r="E83" s="22" t="n"/>
-    </row>
-    <row r="84" ht="18" customHeight="1">
-      <c r="A84" s="21" t="n"/>
-      <c r="E84" s="22" t="n"/>
-    </row>
-    <row r="85" ht="18" customHeight="1">
-      <c r="A85" s="23" t="n"/>
-      <c r="B85" s="24" t="n"/>
-      <c r="C85" s="24" t="n"/>
-      <c r="D85" s="24" t="n"/>
-      <c r="E85" s="25" t="n"/>
+      <c r="B86" s="20" t="n"/>
+      <c r="C86" s="20" t="n"/>
+      <c r="D86" s="20" t="n"/>
+      <c r="E86" s="21" t="n"/>
     </row>
     <row r="87" ht="18" customHeight="1">
-      <c r="A87" s="2" t="inlineStr">
+      <c r="A87" s="18" t="n"/>
+      <c r="B87" s="22" t="n"/>
+      <c r="C87" s="22" t="n"/>
+      <c r="D87" s="22" t="n"/>
+      <c r="E87" s="23" t="n"/>
+    </row>
+    <row r="88" ht="18" customHeight="1">
+      <c r="A88" s="24" t="n"/>
+      <c r="E88" s="25" t="n"/>
+    </row>
+    <row r="89" ht="18" customHeight="1">
+      <c r="A89" s="24" t="n"/>
+      <c r="E89" s="25" t="n"/>
+    </row>
+    <row r="90" ht="18" customHeight="1">
+      <c r="A90" s="24" t="n"/>
+      <c r="E90" s="25" t="n"/>
+    </row>
+    <row r="91" ht="18" customHeight="1">
+      <c r="A91" s="26" t="n"/>
+      <c r="B91" s="27" t="n"/>
+      <c r="C91" s="27" t="n"/>
+      <c r="D91" s="27" t="n"/>
+      <c r="E91" s="28" t="n"/>
+    </row>
+    <row r="93" ht="18" customHeight="1">
+      <c r="A93" s="2" t="inlineStr">
         <is>
           <t>10.  SIGN-OFF</t>
         </is>
       </c>
-      <c r="B87" s="17" t="n"/>
-      <c r="C87" s="17" t="n"/>
-      <c r="D87" s="17" t="n"/>
-      <c r="E87" s="18" t="n"/>
-    </row>
-    <row r="88" ht="28" customHeight="1">
-      <c r="A88" s="6" t="inlineStr">
+      <c r="B93" s="20" t="n"/>
+      <c r="C93" s="20" t="n"/>
+      <c r="D93" s="20" t="n"/>
+      <c r="E93" s="21" t="n"/>
+    </row>
+    <row r="94" ht="28" customHeight="1">
+      <c r="A94" s="6" t="inlineStr">
         <is>
           <t>Role</t>
         </is>
       </c>
-      <c r="B88" s="6" t="inlineStr">
+      <c r="B94" s="6" t="inlineStr">
         <is>
           <t>Name (print)</t>
         </is>
       </c>
-      <c r="C88" s="6" t="inlineStr">
+      <c r="C94" s="6" t="inlineStr">
         <is>
           <t>Signature</t>
         </is>
       </c>
-      <c r="D88" s="6" t="inlineStr">
+      <c r="D94" s="6" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="E88" s="18" t="n"/>
-    </row>
-    <row r="89" ht="24" customHeight="1">
-      <c r="A89" s="3" t="inlineStr">
+      <c r="E94" s="21" t="n"/>
+    </row>
+    <row r="95" ht="24" customHeight="1">
+      <c r="A95" s="3" t="inlineStr">
         <is>
           <t>Technician</t>
         </is>
       </c>
-      <c r="B89" s="4" t="n"/>
-      <c r="C89" s="4" t="n"/>
-      <c r="D89" s="4" t="n"/>
-      <c r="E89" s="18" t="n"/>
-    </row>
-    <row r="90" ht="24" customHeight="1">
-      <c r="A90" s="3" t="inlineStr">
+      <c r="B95" s="4" t="n"/>
+      <c r="C95" s="4" t="n"/>
+      <c r="D95" s="4" t="n"/>
+      <c r="E95" s="21" t="n"/>
+    </row>
+    <row r="96" ht="24" customHeight="1">
+      <c r="A96" s="3" t="inlineStr">
         <is>
           <t>Supervisor / Witness</t>
         </is>
       </c>
-      <c r="B90" s="4" t="n"/>
-      <c r="C90" s="4" t="n"/>
-      <c r="D90" s="4" t="n"/>
-      <c r="E90" s="18" t="n"/>
+      <c r="B96" s="4" t="n"/>
+      <c r="C96" s="4" t="n"/>
+      <c r="D96" s="4" t="n"/>
+      <c r="E96" s="21" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="54">
     <mergeCell ref="A30:E30"/>
-    <mergeCell ref="D69:E69"/>
-    <mergeCell ref="A81:E85"/>
     <mergeCell ref="D60:E60"/>
     <mergeCell ref="B9:E9"/>
-    <mergeCell ref="A48:E48"/>
-    <mergeCell ref="A73:E73"/>
     <mergeCell ref="A15:E15"/>
-    <mergeCell ref="D90:E90"/>
+    <mergeCell ref="D63:E63"/>
     <mergeCell ref="B6:E6"/>
-    <mergeCell ref="A49:E49"/>
+    <mergeCell ref="D81:E81"/>
     <mergeCell ref="A1:E1"/>
+    <mergeCell ref="D84:E84"/>
     <mergeCell ref="B5:E5"/>
-    <mergeCell ref="B63:E63"/>
+    <mergeCell ref="D65:E65"/>
+    <mergeCell ref="D96:E96"/>
+    <mergeCell ref="A79:E79"/>
     <mergeCell ref="D77:E77"/>
-    <mergeCell ref="A87:E87"/>
-    <mergeCell ref="D52:E52"/>
-    <mergeCell ref="A65:E65"/>
+    <mergeCell ref="D95:E95"/>
     <mergeCell ref="B4:E4"/>
+    <mergeCell ref="A54:E54"/>
     <mergeCell ref="D57:E57"/>
     <mergeCell ref="D76:E76"/>
-    <mergeCell ref="A41:E41"/>
     <mergeCell ref="B16:E16"/>
     <mergeCell ref="B7:E7"/>
     <mergeCell ref="D61:E61"/>
-    <mergeCell ref="A66:E66"/>
-    <mergeCell ref="D70:E70"/>
-    <mergeCell ref="A74:E74"/>
+    <mergeCell ref="D66:E66"/>
     <mergeCell ref="A80:E80"/>
     <mergeCell ref="A18:E18"/>
     <mergeCell ref="D75:E75"/>
     <mergeCell ref="A3:E3"/>
-    <mergeCell ref="D53:E53"/>
-    <mergeCell ref="D78:E78"/>
+    <mergeCell ref="A87:E91"/>
+    <mergeCell ref="A55:E55"/>
+    <mergeCell ref="A86:E86"/>
     <mergeCell ref="B12:E12"/>
+    <mergeCell ref="A71:E71"/>
+    <mergeCell ref="A47:E47"/>
     <mergeCell ref="B11:E11"/>
     <mergeCell ref="D62:E62"/>
     <mergeCell ref="A14:E14"/>
     <mergeCell ref="D56:E56"/>
     <mergeCell ref="D58:E58"/>
-    <mergeCell ref="D71:E71"/>
+    <mergeCell ref="D83:E83"/>
     <mergeCell ref="A29:E29"/>
+    <mergeCell ref="D74:E74"/>
     <mergeCell ref="B8:E8"/>
-    <mergeCell ref="D55:E55"/>
     <mergeCell ref="D68:E68"/>
+    <mergeCell ref="D64:E64"/>
+    <mergeCell ref="A72:E72"/>
+    <mergeCell ref="D82:E82"/>
     <mergeCell ref="D67:E67"/>
-    <mergeCell ref="D88:E88"/>
-    <mergeCell ref="D51:E51"/>
+    <mergeCell ref="B69:E69"/>
+    <mergeCell ref="D73:E73"/>
     <mergeCell ref="A19:E19"/>
-    <mergeCell ref="D89:E89"/>
-    <mergeCell ref="D54:E54"/>
-    <mergeCell ref="D50:E50"/>
+    <mergeCell ref="A93:E93"/>
+    <mergeCell ref="D94:E94"/>
     <mergeCell ref="B10:E10"/>
     <mergeCell ref="D59:E59"/>
   </mergeCells>

</xml_diff>

<commit_message>
Split ABB biennial into separate 670 and 615 files; rebrand all templates
Replace ABB_Biennial_Visual_Check.xlsx (2-tab combined) with two standalone
files: ABB_670_Biennial_Visual_Check.xlsx (REG670/RET670) and
ABB_615_Biennial_Visual_Check.xlsx (REF/RET/REM/REU615). Split because the
670 and 615 front-panel workflows, self-supervision signals, and measurement
labels differ enough to be confusing in a shared form.

Also: add LibreOffice lock file pattern to .gitignore; update CLAUDE.md to
document the 3-file biennial structure; rebrand all xlsx templates.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SEL_Biennial_Visual_Check.xlsx
+++ b/SEL_Biennial_Visual_Check.xlsx
@@ -250,7 +250,10 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="53">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -673,1199 +676,1199 @@
   <dimension ref="A1:E96"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="30" customWidth="1" style="21" min="1" max="1"/>
-    <col width="32" customWidth="1" style="21" min="2" max="2"/>
-    <col width="14" customWidth="1" style="21" min="3" max="4"/>
-    <col width="12" customWidth="1" style="21" min="5" max="5"/>
+    <col width="30" customWidth="1" style="22" min="1" max="1"/>
+    <col width="32" customWidth="1" style="22" min="2" max="2"/>
+    <col width="14" customWidth="1" style="22" min="3" max="4"/>
+    <col width="12" customWidth="1" style="22" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="27.75" customHeight="1" s="22">
-      <c r="A1" s="23" t="inlineStr">
+    <row r="1" ht="27.75" customHeight="1" s="23">
+      <c r="A1" s="24" t="inlineStr">
         <is>
           <t>SEL PROTECTION RELAY — BIENNIAL (2-YEARLY) VISUAL CHECK SHEET</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="18" customHeight="1" s="22">
-      <c r="A3" s="24" t="inlineStr">
+    <row r="3" ht="18" customHeight="1" s="23">
+      <c r="A3" s="25" t="inlineStr">
         <is>
           <t>1.  RELAY AND SITE INFORMATION</t>
         </is>
       </c>
-      <c r="B3" s="25" t="n"/>
-      <c r="C3" s="25" t="n"/>
-      <c r="D3" s="25" t="n"/>
-      <c r="E3" s="26" t="n"/>
-    </row>
-    <row r="4" ht="15" customHeight="1" s="22">
-      <c r="A4" s="27" t="inlineStr">
+      <c r="B3" s="26" t="n"/>
+      <c r="C3" s="26" t="n"/>
+      <c r="D3" s="26" t="n"/>
+      <c r="E3" s="27" t="n"/>
+    </row>
+    <row r="4" ht="15" customHeight="1" s="23">
+      <c r="A4" s="28" t="inlineStr">
         <is>
           <t>Relay Model</t>
         </is>
       </c>
-      <c r="B4" s="28" t="inlineStr">
+      <c r="B4" s="29" t="inlineStr">
         <is>
           <t>SEL-300G  /  SEL-311L  /  SEL-787  /  SEL-700G  (circle one)</t>
         </is>
       </c>
-      <c r="C4" s="25" t="n"/>
-      <c r="D4" s="25" t="n"/>
-      <c r="E4" s="26" t="n"/>
-    </row>
-    <row r="5" ht="15" customHeight="1" s="22">
-      <c r="A5" s="27" t="inlineStr">
+      <c r="C4" s="26" t="n"/>
+      <c r="D4" s="26" t="n"/>
+      <c r="E4" s="27" t="n"/>
+    </row>
+    <row r="5" ht="15" customHeight="1" s="23">
+      <c r="A5" s="28" t="inlineStr">
         <is>
           <t>Protected Equipment</t>
         </is>
       </c>
-      <c r="B5" s="28" t="n"/>
-      <c r="C5" s="25" t="n"/>
-      <c r="D5" s="25" t="n"/>
-      <c r="E5" s="26" t="n"/>
-    </row>
-    <row r="6" ht="15" customHeight="1" s="22">
-      <c r="A6" s="27" t="inlineStr">
+      <c r="B5" s="29" t="n"/>
+      <c r="C5" s="26" t="n"/>
+      <c r="D5" s="26" t="n"/>
+      <c r="E5" s="27" t="n"/>
+    </row>
+    <row r="6" ht="15" customHeight="1" s="23">
+      <c r="A6" s="28" t="inlineStr">
         <is>
           <t>Site / Substation</t>
         </is>
       </c>
-      <c r="B6" s="28" t="n"/>
-      <c r="C6" s="25" t="n"/>
-      <c r="D6" s="25" t="n"/>
-      <c r="E6" s="26" t="n"/>
-    </row>
-    <row r="7" ht="15" customHeight="1" s="22">
-      <c r="A7" s="27" t="inlineStr">
+      <c r="B6" s="29" t="n"/>
+      <c r="C6" s="26" t="n"/>
+      <c r="D6" s="26" t="n"/>
+      <c r="E6" s="27" t="n"/>
+    </row>
+    <row r="7" ht="15" customHeight="1" s="23">
+      <c r="A7" s="28" t="inlineStr">
         <is>
           <t>Relay ID (RID / TID)</t>
         </is>
       </c>
-      <c r="B7" s="28" t="n"/>
-      <c r="C7" s="25" t="n"/>
-      <c r="D7" s="25" t="n"/>
-      <c r="E7" s="26" t="n"/>
-    </row>
-    <row r="8" ht="15" customHeight="1" s="22">
-      <c r="A8" s="27" t="inlineStr">
+      <c r="B7" s="29" t="n"/>
+      <c r="C7" s="26" t="n"/>
+      <c r="D7" s="26" t="n"/>
+      <c r="E7" s="27" t="n"/>
+    </row>
+    <row r="8" ht="15" customHeight="1" s="23">
+      <c r="A8" s="28" t="inlineStr">
         <is>
           <t>Panel / Cubicle Tag</t>
         </is>
       </c>
-      <c r="B8" s="28" t="n"/>
-      <c r="C8" s="25" t="n"/>
-      <c r="D8" s="25" t="n"/>
-      <c r="E8" s="26" t="n"/>
-    </row>
-    <row r="9" ht="15" customHeight="1" s="22">
-      <c r="A9" s="27" t="inlineStr">
+      <c r="B8" s="29" t="n"/>
+      <c r="C8" s="26" t="n"/>
+      <c r="D8" s="26" t="n"/>
+      <c r="E8" s="27" t="n"/>
+    </row>
+    <row r="9" ht="15" customHeight="1" s="23">
+      <c r="A9" s="28" t="inlineStr">
         <is>
           <t>Work Order No.</t>
         </is>
       </c>
-      <c r="B9" s="28" t="n"/>
-      <c r="C9" s="25" t="n"/>
-      <c r="D9" s="25" t="n"/>
-      <c r="E9" s="26" t="n"/>
-    </row>
-    <row r="10" ht="15" customHeight="1" s="22">
-      <c r="A10" s="27" t="inlineStr">
+      <c r="B9" s="29" t="n"/>
+      <c r="C9" s="26" t="n"/>
+      <c r="D9" s="26" t="n"/>
+      <c r="E9" s="27" t="n"/>
+    </row>
+    <row r="10" ht="15" customHeight="1" s="23">
+      <c r="A10" s="28" t="inlineStr">
         <is>
           <t>Date of Check</t>
         </is>
       </c>
-      <c r="B10" s="28" t="n"/>
-      <c r="C10" s="25" t="n"/>
-      <c r="D10" s="25" t="n"/>
-      <c r="E10" s="26" t="n"/>
-    </row>
-    <row r="11" ht="15" customHeight="1" s="22">
-      <c r="A11" s="27" t="inlineStr">
+      <c r="B10" s="29" t="n"/>
+      <c r="C10" s="26" t="n"/>
+      <c r="D10" s="26" t="n"/>
+      <c r="E10" s="27" t="n"/>
+    </row>
+    <row r="11" ht="15" customHeight="1" s="23">
+      <c r="A11" s="28" t="inlineStr">
         <is>
           <t>Technician Name</t>
         </is>
       </c>
-      <c r="B11" s="28" t="n"/>
-      <c r="C11" s="25" t="n"/>
-      <c r="D11" s="25" t="n"/>
-      <c r="E11" s="26" t="n"/>
-    </row>
-    <row r="12" ht="15" customHeight="1" s="22">
-      <c r="A12" s="27" t="inlineStr">
+      <c r="B11" s="29" t="n"/>
+      <c r="C11" s="26" t="n"/>
+      <c r="D11" s="26" t="n"/>
+      <c r="E11" s="27" t="n"/>
+    </row>
+    <row r="12" ht="15" customHeight="1" s="23">
+      <c r="A12" s="28" t="inlineStr">
         <is>
           <t>Next Check Due</t>
         </is>
       </c>
-      <c r="B12" s="28" t="inlineStr">
+      <c r="B12" s="29" t="inlineStr">
         <is>
           <t>(2 years from date above)</t>
         </is>
       </c>
-      <c r="C12" s="25" t="n"/>
-      <c r="D12" s="25" t="n"/>
-      <c r="E12" s="26" t="n"/>
-    </row>
-    <row r="14" ht="18" customHeight="1" s="22">
-      <c r="A14" s="24" t="inlineStr">
+      <c r="C12" s="26" t="n"/>
+      <c r="D12" s="26" t="n"/>
+      <c r="E12" s="27" t="n"/>
+    </row>
+    <row r="14" ht="18" customHeight="1" s="23">
+      <c r="A14" s="25" t="inlineStr">
         <is>
           <t>2.  CONNECTION METHOD</t>
         </is>
       </c>
-      <c r="B14" s="25" t="n"/>
-      <c r="C14" s="25" t="n"/>
-      <c r="D14" s="25" t="n"/>
-      <c r="E14" s="26" t="n"/>
-    </row>
-    <row r="15" ht="51.75" customHeight="1" s="22">
-      <c r="A15" s="29" t="inlineStr">
+      <c r="B14" s="26" t="n"/>
+      <c r="C14" s="26" t="n"/>
+      <c r="D14" s="26" t="n"/>
+      <c r="E14" s="27" t="n"/>
+    </row>
+    <row r="15" ht="51.75" customHeight="1" s="23">
+      <c r="A15" s="30" t="inlineStr">
         <is>
           <t>OPTION A — Front panel only (no laptop): Press any key to wake display. Navigate with arrow keys.
 OPTION B — Serial cable: Connect SEL-C662 cable (laptop USB → relay front DB-9). Open PuTTY/terminal: 19200 baud, 8-N-1, no flow control. Press Enter → prompt appears. Type ACC &lt;Enter&gt;, enter Level 1 password (default: OTTER).
 OPTION C — Ethernet (if fitted): Open AcSELerator QuickSet or SSH/Telnet to relay IP.</t>
         </is>
       </c>
-      <c r="B15" s="25" t="n"/>
-      <c r="C15" s="25" t="n"/>
-      <c r="D15" s="25" t="n"/>
-      <c r="E15" s="26" t="n"/>
-    </row>
-    <row r="16" ht="15" customHeight="1" s="22">
-      <c r="A16" s="27" t="inlineStr">
+      <c r="B15" s="26" t="n"/>
+      <c r="C15" s="26" t="n"/>
+      <c r="D15" s="26" t="n"/>
+      <c r="E15" s="27" t="n"/>
+    </row>
+    <row r="16" ht="15" customHeight="1" s="23">
+      <c r="A16" s="28" t="inlineStr">
         <is>
           <t>Connection method used today</t>
         </is>
       </c>
-      <c r="B16" s="28" t="inlineStr">
+      <c r="B16" s="29" t="inlineStr">
         <is>
           <t>Front panel / Serial cable / Ethernet  (delete as applicable)</t>
         </is>
       </c>
-      <c r="C16" s="25" t="n"/>
-      <c r="D16" s="25" t="n"/>
-      <c r="E16" s="26" t="n"/>
-    </row>
-    <row r="18" ht="18" customHeight="1" s="22">
-      <c r="A18" s="24" t="inlineStr">
+      <c r="C16" s="26" t="n"/>
+      <c r="D16" s="26" t="n"/>
+      <c r="E16" s="27" t="n"/>
+    </row>
+    <row r="18" ht="18" customHeight="1" s="23">
+      <c r="A18" s="25" t="inlineStr">
         <is>
           <t>3.  SELF-TEST AND DEVICE STATUS</t>
         </is>
       </c>
-      <c r="B18" s="25" t="n"/>
-      <c r="C18" s="25" t="n"/>
-      <c r="D18" s="25" t="n"/>
-      <c r="E18" s="26" t="n"/>
-    </row>
-    <row r="19" ht="36" customHeight="1" s="22">
-      <c r="A19" s="29" t="inlineStr">
+      <c r="B18" s="26" t="n"/>
+      <c r="C18" s="26" t="n"/>
+      <c r="D18" s="26" t="n"/>
+      <c r="E18" s="27" t="n"/>
+    </row>
+    <row r="19" ht="36" customHeight="1" s="23">
+      <c r="A19" s="30" t="inlineStr">
         <is>
           <t>Front panel: ENABLED LED (green, solid) must be illuminated. Serial: type STA &lt;Enter&gt; or STATUS &lt;Enter&gt; — all items should show OK. W = warning (issue STA C to clear), FAIL = fault (requires investigation).</t>
         </is>
       </c>
-      <c r="B19" s="25" t="n"/>
-      <c r="C19" s="25" t="n"/>
-      <c r="D19" s="25" t="n"/>
-      <c r="E19" s="26" t="n"/>
-    </row>
-    <row r="20" ht="27.75" customHeight="1" s="22">
-      <c r="A20" s="30" t="inlineStr">
+      <c r="B19" s="26" t="n"/>
+      <c r="C19" s="26" t="n"/>
+      <c r="D19" s="26" t="n"/>
+      <c r="E19" s="27" t="n"/>
+    </row>
+    <row r="20" ht="27.75" customHeight="1" s="23">
+      <c r="A20" s="31" t="inlineStr">
         <is>
           <t>Check Item</t>
         </is>
       </c>
-      <c r="B20" s="30" t="inlineStr">
+      <c r="B20" s="31" t="inlineStr">
         <is>
           <t>How to Read / Where to Look</t>
         </is>
       </c>
-      <c r="C20" s="30" t="inlineStr">
+      <c r="C20" s="31" t="inlineStr">
         <is>
           <t>Expected</t>
         </is>
       </c>
-      <c r="D20" s="30" t="inlineStr">
+      <c r="D20" s="31" t="inlineStr">
         <is>
           <t>Result</t>
         </is>
       </c>
-      <c r="E20" s="30" t="inlineStr">
+      <c r="E20" s="31" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="15" customHeight="1" s="22">
-      <c r="A21" s="31" t="inlineStr">
+    <row r="21" ht="15" customHeight="1" s="23">
+      <c r="A21" s="32" t="inlineStr">
         <is>
           <t>ENABLED LED (green, solid)</t>
         </is>
       </c>
-      <c r="B21" s="32" t="inlineStr">
+      <c r="B21" s="33" t="inlineStr">
         <is>
           <t>Visual — front panel top-right LED</t>
         </is>
       </c>
-      <c r="C21" s="33" t="inlineStr">
+      <c r="C21" s="34" t="inlineStr">
         <is>
           <t>ON (solid green)</t>
         </is>
       </c>
-      <c r="D21" s="34" t="n"/>
-      <c r="E21" s="28" t="n"/>
-    </row>
-    <row r="22" ht="15" customHeight="1" s="22">
-      <c r="A22" s="31" t="inlineStr">
+      <c r="D21" s="35" t="n"/>
+      <c r="E21" s="29" t="n"/>
+    </row>
+    <row r="22" ht="15" customHeight="1" s="23">
+      <c r="A22" s="32" t="inlineStr">
         <is>
           <t>No alarm LEDs active</t>
         </is>
       </c>
-      <c r="B22" s="32" t="inlineStr">
+      <c r="B22" s="33" t="inlineStr">
         <is>
           <t>Visual — front panel LEDs</t>
         </is>
       </c>
-      <c r="C22" s="33" t="inlineStr">
+      <c r="C22" s="34" t="inlineStr">
         <is>
           <t>All alarm LEDs off</t>
         </is>
       </c>
-      <c r="D22" s="34" t="n"/>
-      <c r="E22" s="28" t="n"/>
-    </row>
-    <row r="23" ht="15" customHeight="1" s="22">
-      <c r="A23" s="31" t="inlineStr">
+      <c r="D22" s="35" t="n"/>
+      <c r="E22" s="29" t="n"/>
+    </row>
+    <row r="23" ht="15" customHeight="1" s="23">
+      <c r="A23" s="32" t="inlineStr">
         <is>
           <t>Front panel display</t>
         </is>
       </c>
-      <c r="B23" s="32" t="inlineStr">
+      <c r="B23" s="33" t="inlineStr">
         <is>
           <t>Visual — press any key to wake</t>
         </is>
       </c>
-      <c r="C23" s="33" t="inlineStr">
+      <c r="C23" s="34" t="inlineStr">
         <is>
           <t>No error messages shown</t>
         </is>
       </c>
-      <c r="D23" s="34" t="n"/>
-      <c r="E23" s="28" t="n"/>
-    </row>
-    <row r="24" ht="20.85" customHeight="1" s="22">
-      <c r="A24" s="31" t="inlineStr">
+      <c r="D23" s="35" t="n"/>
+      <c r="E23" s="29" t="n"/>
+    </row>
+    <row r="24" ht="20.25" customHeight="1" s="23">
+      <c r="A24" s="32" t="inlineStr">
         <is>
           <t>Self-test status — all OK</t>
         </is>
       </c>
-      <c r="B24" s="32" t="inlineStr">
+      <c r="B24" s="33" t="inlineStr">
         <is>
           <t>Serial: STA &lt;Enter&gt;
 Front panel: Main &gt; Status</t>
         </is>
       </c>
-      <c r="C24" s="33" t="inlineStr">
+      <c r="C24" s="34" t="inlineStr">
         <is>
           <t>All items = OK</t>
         </is>
       </c>
-      <c r="D24" s="34" t="n"/>
-      <c r="E24" s="28" t="n"/>
-    </row>
-    <row r="25" ht="15" customHeight="1" s="22">
-      <c r="A25" s="31" t="inlineStr">
+      <c r="D24" s="35" t="n"/>
+      <c r="E24" s="29" t="n"/>
+    </row>
+    <row r="25" ht="15" customHeight="1" s="23">
+      <c r="A25" s="32" t="inlineStr">
         <is>
           <t>HALARM bit (hardware alarm)</t>
         </is>
       </c>
-      <c r="B25" s="32" t="inlineStr">
+      <c r="B25" s="33" t="inlineStr">
         <is>
           <t>STA output: look for HALARM = 0</t>
         </is>
       </c>
-      <c r="C25" s="33" t="inlineStr">
+      <c r="C25" s="34" t="inlineStr">
         <is>
           <t>0 (not asserted)</t>
         </is>
       </c>
-      <c r="D25" s="34" t="n"/>
-      <c r="E25" s="28" t="n"/>
-    </row>
-    <row r="26" ht="15" customHeight="1" s="22">
-      <c r="A26" s="31" t="inlineStr">
+      <c r="D25" s="35" t="n"/>
+      <c r="E25" s="29" t="n"/>
+    </row>
+    <row r="26" ht="15" customHeight="1" s="23">
+      <c r="A26" s="32" t="inlineStr">
         <is>
           <t>SALARM bit (software alarm)</t>
         </is>
       </c>
-      <c r="B26" s="32" t="inlineStr">
+      <c r="B26" s="33" t="inlineStr">
         <is>
           <t>STA output: look for SALARM = 0</t>
         </is>
       </c>
-      <c r="C26" s="33" t="inlineStr">
+      <c r="C26" s="34" t="inlineStr">
         <is>
           <t>0 (not asserted)</t>
         </is>
       </c>
-      <c r="D26" s="34" t="n"/>
-      <c r="E26" s="28" t="n"/>
-    </row>
-    <row r="27" ht="15" customHeight="1" s="22">
-      <c r="A27" s="31" t="inlineStr">
+      <c r="D26" s="35" t="n"/>
+      <c r="E26" s="29" t="n"/>
+    </row>
+    <row r="27" ht="15" customHeight="1" s="23">
+      <c r="A27" s="32" t="inlineStr">
         <is>
           <t>Relay shows 'Relay Enabled'</t>
         </is>
       </c>
-      <c r="B27" s="32" t="inlineStr">
+      <c r="B27" s="33" t="inlineStr">
         <is>
           <t>Last line of STA output</t>
         </is>
       </c>
-      <c r="C27" s="33" t="inlineStr">
+      <c r="C27" s="34" t="inlineStr">
         <is>
           <t>'Relay Enabled'</t>
         </is>
       </c>
-      <c r="D27" s="34" t="n"/>
-      <c r="E27" s="28" t="n"/>
-    </row>
-    <row r="29" ht="18" customHeight="1" s="22">
-      <c r="A29" s="24" t="inlineStr">
+      <c r="D27" s="35" t="n"/>
+      <c r="E27" s="29" t="n"/>
+    </row>
+    <row r="29" ht="18" customHeight="1" s="23">
+      <c r="A29" s="25" t="inlineStr">
         <is>
           <t>4.  ANALOGUE MEASUREMENTS  (Primary Values — relay reports in primary units)</t>
         </is>
       </c>
-      <c r="B29" s="25" t="n"/>
-      <c r="C29" s="25" t="n"/>
-      <c r="D29" s="25" t="n"/>
-      <c r="E29" s="26" t="n"/>
-    </row>
-    <row r="30" ht="39.75" customHeight="1" s="22">
-      <c r="A30" s="29" t="inlineStr">
+      <c r="B29" s="26" t="n"/>
+      <c r="C29" s="26" t="n"/>
+      <c r="D29" s="26" t="n"/>
+      <c r="E29" s="27" t="n"/>
+    </row>
+    <row r="30" ht="39.75" customHeight="1" s="23">
+      <c r="A30" s="30" t="inlineStr">
         <is>
           <t>Serial: type METER &lt;Enter&gt; — relay displays primary values (A and V). Front panel: Main &gt; Meters &gt; Fundamental.  Record measured values. Compare to expected load (no specific pass/fail for 2-yearly — flag anything obviously wrong, e.g., one phase zero when others are normal).</t>
         </is>
       </c>
-      <c r="B30" s="25" t="n"/>
-      <c r="C30" s="25" t="n"/>
-      <c r="D30" s="25" t="n"/>
-      <c r="E30" s="26" t="n"/>
-    </row>
-    <row r="31" ht="27.75" customHeight="1" s="22">
-      <c r="A31" s="30" t="inlineStr">
+      <c r="B30" s="26" t="n"/>
+      <c r="C30" s="26" t="n"/>
+      <c r="D30" s="26" t="n"/>
+      <c r="E30" s="27" t="n"/>
+    </row>
+    <row r="31" ht="27.75" customHeight="1" s="23">
+      <c r="A31" s="31" t="inlineStr">
         <is>
           <t>Quantity</t>
         </is>
       </c>
-      <c r="B31" s="30" t="inlineStr">
+      <c r="B31" s="31" t="inlineStr">
         <is>
           <t>Reading Method</t>
         </is>
       </c>
-      <c r="C31" s="30" t="inlineStr">
+      <c r="C31" s="31" t="inlineStr">
         <is>
           <t>Measured Value</t>
         </is>
       </c>
-      <c r="D31" s="30" t="inlineStr">
+      <c r="D31" s="31" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="E31" s="30" t="inlineStr">
+      <c r="E31" s="31" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="15" customHeight="1" s="22">
-      <c r="A32" s="31" t="inlineStr">
+    <row r="32" ht="15" customHeight="1" s="23">
+      <c r="A32" s="32" t="inlineStr">
         <is>
           <t>IA — Phase A Current (primary)</t>
         </is>
       </c>
-      <c r="B32" s="32" t="inlineStr">
+      <c r="B32" s="33" t="inlineStr">
         <is>
           <t>METER / Meters &gt; Fundamental</t>
         </is>
       </c>
-      <c r="C32" s="34" t="n"/>
-      <c r="D32" s="35" t="inlineStr">
+      <c r="C32" s="35" t="n"/>
+      <c r="D32" s="36" t="inlineStr">
         <is>
           <t>A primary</t>
         </is>
       </c>
-      <c r="E32" s="28" t="n"/>
-    </row>
-    <row r="33" ht="15" customHeight="1" s="22">
-      <c r="A33" s="31" t="inlineStr">
+      <c r="E32" s="29" t="n"/>
+    </row>
+    <row r="33" ht="15" customHeight="1" s="23">
+      <c r="A33" s="32" t="inlineStr">
         <is>
           <t>IB — Phase B Current (primary)</t>
         </is>
       </c>
-      <c r="B33" s="32" t="inlineStr">
+      <c r="B33" s="33" t="inlineStr">
         <is>
           <t>METER / Meters &gt; Fundamental</t>
         </is>
       </c>
-      <c r="C33" s="34" t="n"/>
-      <c r="D33" s="35" t="inlineStr">
+      <c r="C33" s="35" t="n"/>
+      <c r="D33" s="36" t="inlineStr">
         <is>
           <t>A primary</t>
         </is>
       </c>
-      <c r="E33" s="28" t="n"/>
-    </row>
-    <row r="34" ht="15" customHeight="1" s="22">
-      <c r="A34" s="31" t="inlineStr">
+      <c r="E33" s="29" t="n"/>
+    </row>
+    <row r="34" ht="15" customHeight="1" s="23">
+      <c r="A34" s="32" t="inlineStr">
         <is>
           <t>IC — Phase C Current (primary)</t>
         </is>
       </c>
-      <c r="B34" s="32" t="inlineStr">
+      <c r="B34" s="33" t="inlineStr">
         <is>
           <t>METER / Meters &gt; Fundamental</t>
         </is>
       </c>
-      <c r="C34" s="34" t="n"/>
-      <c r="D34" s="35" t="inlineStr">
+      <c r="C34" s="35" t="n"/>
+      <c r="D34" s="36" t="inlineStr">
         <is>
           <t>A primary</t>
         </is>
       </c>
-      <c r="E34" s="28" t="n"/>
-    </row>
-    <row r="35" ht="15" customHeight="1" s="22">
-      <c r="A35" s="31" t="inlineStr">
+      <c r="E34" s="29" t="n"/>
+    </row>
+    <row r="35" ht="15" customHeight="1" s="23">
+      <c r="A35" s="32" t="inlineStr">
         <is>
           <t>IN / IGX — Residual / Neutral</t>
         </is>
       </c>
-      <c r="B35" s="32" t="inlineStr">
+      <c r="B35" s="33" t="inlineStr">
         <is>
           <t>METER / Meters &gt; Fundamental</t>
         </is>
       </c>
-      <c r="C35" s="34" t="n"/>
-      <c r="D35" s="35" t="inlineStr">
+      <c r="C35" s="35" t="n"/>
+      <c r="D35" s="36" t="inlineStr">
         <is>
           <t>A primary</t>
         </is>
       </c>
-      <c r="E35" s="28" t="n"/>
-    </row>
-    <row r="36" ht="20.85" customHeight="1" s="22">
-      <c r="A36" s="31" t="inlineStr">
+      <c r="E35" s="29" t="n"/>
+    </row>
+    <row r="36" ht="20.25" customHeight="1" s="23">
+      <c r="A36" s="32" t="inlineStr">
         <is>
           <t>VA — Phase A Voltage (primary)</t>
         </is>
       </c>
-      <c r="B36" s="32" t="inlineStr">
+      <c r="B36" s="33" t="inlineStr">
         <is>
           <t>METER / Meters &gt; Fundamental
 (if VT fitted)</t>
         </is>
       </c>
-      <c r="C36" s="34" t="n"/>
-      <c r="D36" s="35" t="inlineStr">
+      <c r="C36" s="35" t="n"/>
+      <c r="D36" s="36" t="inlineStr">
         <is>
           <t>kV primary</t>
         </is>
       </c>
-      <c r="E36" s="28" t="n"/>
-    </row>
-    <row r="37" ht="20.85" customHeight="1" s="22">
-      <c r="A37" s="31" t="inlineStr">
+      <c r="E36" s="29" t="n"/>
+    </row>
+    <row r="37" ht="20.25" customHeight="1" s="23">
+      <c r="A37" s="32" t="inlineStr">
         <is>
           <t>VB — Phase B Voltage (primary)</t>
         </is>
       </c>
-      <c r="B37" s="32" t="inlineStr">
+      <c r="B37" s="33" t="inlineStr">
         <is>
           <t>METER / Meters &gt; Fundamental
 (if VT fitted)</t>
         </is>
       </c>
-      <c r="C37" s="34" t="n"/>
-      <c r="D37" s="35" t="inlineStr">
+      <c r="C37" s="35" t="n"/>
+      <c r="D37" s="36" t="inlineStr">
         <is>
           <t>kV primary</t>
         </is>
       </c>
-      <c r="E37" s="28" t="n"/>
-    </row>
-    <row r="38" ht="20.85" customHeight="1" s="22">
-      <c r="A38" s="31" t="inlineStr">
+      <c r="E37" s="29" t="n"/>
+    </row>
+    <row r="38" ht="20.25" customHeight="1" s="23">
+      <c r="A38" s="32" t="inlineStr">
         <is>
           <t>VC — Phase C Voltage (primary)</t>
         </is>
       </c>
-      <c r="B38" s="32" t="inlineStr">
+      <c r="B38" s="33" t="inlineStr">
         <is>
           <t>METER / Meters &gt; Fundamental
 (if VT fitted)</t>
         </is>
       </c>
-      <c r="C38" s="34" t="n"/>
-      <c r="D38" s="35" t="inlineStr">
+      <c r="C38" s="35" t="n"/>
+      <c r="D38" s="36" t="inlineStr">
         <is>
           <t>kV primary</t>
         </is>
       </c>
-      <c r="E38" s="28" t="n"/>
-    </row>
-    <row r="39" ht="15" customHeight="1" s="22">
-      <c r="A39" s="31" t="inlineStr">
+      <c r="E38" s="29" t="n"/>
+    </row>
+    <row r="39" ht="15" customHeight="1" s="23">
+      <c r="A39" s="32" t="inlineStr">
         <is>
           <t>Frequency</t>
         </is>
       </c>
-      <c r="B39" s="32" t="inlineStr">
+      <c r="B39" s="33" t="inlineStr">
         <is>
           <t>METER / Meters &gt; Fundamental</t>
         </is>
       </c>
-      <c r="C39" s="34" t="n"/>
-      <c r="D39" s="35" t="inlineStr">
+      <c r="C39" s="35" t="n"/>
+      <c r="D39" s="36" t="inlineStr">
         <is>
           <t>Hz</t>
         </is>
       </c>
-      <c r="E39" s="28" t="n"/>
-    </row>
-    <row r="40" ht="15" customHeight="1" s="22">
-      <c r="A40" s="36" t="n"/>
-      <c r="B40" s="35" t="inlineStr">
+      <c r="E39" s="29" t="n"/>
+    </row>
+    <row r="40" ht="15" customHeight="1" s="23">
+      <c r="A40" s="37" t="n"/>
+      <c r="B40" s="36" t="inlineStr">
         <is>
           <t>METER / Meters &gt; Fundamental</t>
         </is>
       </c>
-      <c r="C40" s="37" t="n"/>
-      <c r="D40" s="38" t="n"/>
-      <c r="E40" s="38" t="n"/>
-    </row>
-    <row r="41" ht="15" customHeight="1" s="22">
-      <c r="A41" s="39" t="n"/>
-      <c r="B41" s="35" t="inlineStr">
+      <c r="C40" s="38" t="n"/>
+      <c r="D40" s="39" t="n"/>
+      <c r="E40" s="39" t="n"/>
+    </row>
+    <row r="41" ht="15" customHeight="1" s="23">
+      <c r="A41" s="40" t="n"/>
+      <c r="B41" s="36" t="inlineStr">
         <is>
           <t>METER / Meters &gt; Fundamental</t>
         </is>
       </c>
-      <c r="C41" s="34" t="n"/>
-      <c r="D41" s="28" t="n"/>
-      <c r="E41" s="28" t="n"/>
-    </row>
-    <row r="42" ht="15" customHeight="1" s="22">
-      <c r="A42" s="36" t="n"/>
-      <c r="B42" s="35" t="inlineStr">
+      <c r="C41" s="35" t="n"/>
+      <c r="D41" s="29" t="n"/>
+      <c r="E41" s="29" t="n"/>
+    </row>
+    <row r="42" ht="15" customHeight="1" s="23">
+      <c r="A42" s="37" t="n"/>
+      <c r="B42" s="36" t="inlineStr">
         <is>
           <t>METER / Meters &gt; Fundamental</t>
         </is>
       </c>
-      <c r="C42" s="37" t="n"/>
-      <c r="D42" s="38" t="n"/>
-      <c r="E42" s="38" t="n"/>
-    </row>
-    <row r="43" ht="15" customHeight="1" s="22">
-      <c r="A43" s="39" t="n"/>
-      <c r="B43" s="35" t="inlineStr">
+      <c r="C42" s="38" t="n"/>
+      <c r="D42" s="39" t="n"/>
+      <c r="E42" s="39" t="n"/>
+    </row>
+    <row r="43" ht="15" customHeight="1" s="23">
+      <c r="A43" s="40" t="n"/>
+      <c r="B43" s="36" t="inlineStr">
         <is>
           <t>METER / Meters &gt; Fundamental</t>
         </is>
       </c>
-      <c r="C43" s="34" t="n"/>
-      <c r="D43" s="28" t="n"/>
-      <c r="E43" s="28" t="n"/>
-    </row>
-    <row r="44" ht="15" customHeight="1" s="22">
-      <c r="A44" s="36" t="n"/>
-      <c r="B44" s="35" t="inlineStr">
+      <c r="C43" s="35" t="n"/>
+      <c r="D43" s="29" t="n"/>
+      <c r="E43" s="29" t="n"/>
+    </row>
+    <row r="44" ht="15" customHeight="1" s="23">
+      <c r="A44" s="37" t="n"/>
+      <c r="B44" s="36" t="inlineStr">
         <is>
           <t>METER / Meters &gt; Fundamental</t>
         </is>
       </c>
-      <c r="C44" s="37" t="n"/>
-      <c r="D44" s="38" t="n"/>
-      <c r="E44" s="38" t="n"/>
-    </row>
-    <row r="45" ht="15" customHeight="1" s="22">
-      <c r="A45" s="39" t="n"/>
-      <c r="B45" s="35" t="inlineStr">
+      <c r="C44" s="38" t="n"/>
+      <c r="D44" s="39" t="n"/>
+      <c r="E44" s="39" t="n"/>
+    </row>
+    <row r="45" ht="15" customHeight="1" s="23">
+      <c r="A45" s="40" t="n"/>
+      <c r="B45" s="36" t="inlineStr">
         <is>
           <t>METER / Meters &gt; Fundamental</t>
         </is>
       </c>
-      <c r="C45" s="34" t="n"/>
-      <c r="D45" s="28" t="n"/>
-      <c r="E45" s="28" t="n"/>
-    </row>
-    <row r="47" ht="18" customHeight="1" s="22">
-      <c r="A47" s="24" t="inlineStr">
+      <c r="C45" s="35" t="n"/>
+      <c r="D45" s="29" t="n"/>
+      <c r="E45" s="29" t="n"/>
+    </row>
+    <row r="47" ht="18" customHeight="1" s="23">
+      <c r="A47" s="25" t="inlineStr">
         <is>
           <t>5.  CLOCK AND TIME SYNCHRONISATION</t>
         </is>
       </c>
-      <c r="B47" s="25" t="n"/>
-      <c r="C47" s="25" t="n"/>
-      <c r="D47" s="25" t="n"/>
-      <c r="E47" s="26" t="n"/>
-    </row>
-    <row r="48" ht="27.75" customHeight="1" s="22">
-      <c r="A48" s="30" t="inlineStr">
+      <c r="B47" s="26" t="n"/>
+      <c r="C47" s="26" t="n"/>
+      <c r="D47" s="26" t="n"/>
+      <c r="E47" s="27" t="n"/>
+    </row>
+    <row r="48" ht="27.75" customHeight="1" s="23">
+      <c r="A48" s="31" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
       </c>
-      <c r="B48" s="30" t="inlineStr">
+      <c r="B48" s="31" t="inlineStr">
         <is>
           <t>How to Read</t>
         </is>
       </c>
-      <c r="C48" s="30" t="inlineStr">
+      <c r="C48" s="31" t="inlineStr">
         <is>
           <t>Relay Value</t>
         </is>
       </c>
-      <c r="D48" s="30" t="inlineStr">
+      <c r="D48" s="31" t="inlineStr">
         <is>
           <t>Reference Value</t>
         </is>
       </c>
-      <c r="E48" s="30" t="inlineStr">
+      <c r="E48" s="31" t="inlineStr">
         <is>
           <t>Difference / Result</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="20.85" customHeight="1" s="22">
-      <c r="A49" s="31" t="inlineStr">
+    <row r="49" ht="20.25" customHeight="1" s="23">
+      <c r="A49" s="32" t="inlineStr">
         <is>
           <t>Relay Date</t>
         </is>
       </c>
-      <c r="B49" s="32" t="inlineStr">
+      <c r="B49" s="33" t="inlineStr">
         <is>
           <t>Serial: DAT &lt;Enter&gt;
 Front panel: Main &gt; Time or Status</t>
         </is>
       </c>
-      <c r="C49" s="34" t="n"/>
-      <c r="D49" s="35" t="inlineStr">
+      <c r="C49" s="35" t="n"/>
+      <c r="D49" s="36" t="inlineStr">
         <is>
           <t>Today's date</t>
         </is>
       </c>
-      <c r="E49" s="28" t="n"/>
-    </row>
-    <row r="50" ht="20.85" customHeight="1" s="22">
-      <c r="A50" s="31" t="inlineStr">
+      <c r="E49" s="29" t="n"/>
+    </row>
+    <row r="50" ht="20.25" customHeight="1" s="23">
+      <c r="A50" s="32" t="inlineStr">
         <is>
           <t>Relay Time</t>
         </is>
       </c>
-      <c r="B50" s="32" t="inlineStr">
+      <c r="B50" s="33" t="inlineStr">
         <is>
           <t>Serial: TIM &lt;Enter&gt;
 Front panel: Main &gt; Time or Status</t>
         </is>
       </c>
-      <c r="C50" s="34" t="n"/>
-      <c r="D50" s="35" t="inlineStr">
+      <c r="C50" s="35" t="n"/>
+      <c r="D50" s="36" t="inlineStr">
         <is>
           <t>GPS/NTP reference</t>
         </is>
       </c>
-      <c r="E50" s="28" t="n"/>
-    </row>
-    <row r="51" ht="15" customHeight="1" s="22">
-      <c r="A51" s="31" t="inlineStr">
+      <c r="E50" s="29" t="n"/>
+    </row>
+    <row r="51" ht="15" customHeight="1" s="23">
+      <c r="A51" s="32" t="inlineStr">
         <is>
           <t>Time source (IRIG-B / NTP / Internal)</t>
         </is>
       </c>
-      <c r="B51" s="32" t="inlineStr">
+      <c r="B51" s="33" t="inlineStr">
         <is>
           <t>Serial: STA &lt;Enter&gt; — look for IRIG-B or NTP line</t>
         </is>
       </c>
-      <c r="C51" s="34" t="n"/>
-      <c r="D51" s="35" t="inlineStr">
+      <c r="C51" s="35" t="n"/>
+      <c r="D51" s="36" t="inlineStr">
         <is>
           <t>IRIG-B preferred</t>
         </is>
       </c>
-      <c r="E51" s="28" t="n"/>
-    </row>
-    <row r="52" ht="15" customHeight="1" s="22">
-      <c r="A52" s="31" t="inlineStr">
+      <c r="E51" s="29" t="n"/>
+    </row>
+    <row r="52" ht="15" customHeight="1" s="23">
+      <c r="A52" s="32" t="inlineStr">
         <is>
           <t>Time difference (accept ≤ 10 s)</t>
         </is>
       </c>
-      <c r="B52" s="32" t="inlineStr">
+      <c r="B52" s="33" t="inlineStr">
         <is>
           <t>Relay time vs phone/GPS reference</t>
         </is>
       </c>
-      <c r="C52" s="34" t="n"/>
-      <c r="D52" s="35" t="inlineStr">
+      <c r="C52" s="35" t="n"/>
+      <c r="D52" s="36" t="inlineStr">
         <is>
           <t>≤ 10 s</t>
         </is>
       </c>
-      <c r="E52" s="28" t="n"/>
-    </row>
-    <row r="54" ht="18" customHeight="1" s="22">
-      <c r="A54" s="24" t="inlineStr">
+      <c r="E52" s="29" t="n"/>
+    </row>
+    <row r="54" ht="18" customHeight="1" s="23">
+      <c r="A54" s="25" t="inlineStr">
         <is>
           <t>6.  RECENT EVENTS  (record most recent events — flag any unexplained trips or alarms)</t>
         </is>
       </c>
-      <c r="B54" s="25" t="n"/>
-      <c r="C54" s="25" t="n"/>
-      <c r="D54" s="25" t="n"/>
-      <c r="E54" s="26" t="n"/>
-    </row>
-    <row r="55" ht="36" customHeight="1" s="22">
-      <c r="A55" s="29" t="inlineStr">
+      <c r="B54" s="26" t="n"/>
+      <c r="C54" s="26" t="n"/>
+      <c r="D54" s="26" t="n"/>
+      <c r="E54" s="27" t="n"/>
+    </row>
+    <row r="55" ht="36" customHeight="1" s="23">
+      <c r="A55" s="30" t="inlineStr">
         <is>
           <t>Serial: type HIS &lt;Enter&gt; for event history, or EVE &lt;Enter&gt; for last event report, or SER &lt;Enter&gt; for Sequential Events Recorder.  Front panel: Main &gt; Events (or Main &gt; Targets for relay word bits).  Record the most recent events and their dates below.</t>
         </is>
       </c>
-      <c r="B55" s="25" t="n"/>
-      <c r="C55" s="25" t="n"/>
-      <c r="D55" s="25" t="n"/>
-      <c r="E55" s="26" t="n"/>
-    </row>
-    <row r="56" ht="27.75" customHeight="1" s="22">
-      <c r="A56" s="30" t="inlineStr">
+      <c r="B55" s="26" t="n"/>
+      <c r="C55" s="26" t="n"/>
+      <c r="D55" s="26" t="n"/>
+      <c r="E55" s="27" t="n"/>
+    </row>
+    <row r="56" ht="27.75" customHeight="1" s="23">
+      <c r="A56" s="31" t="inlineStr">
         <is>
           <t>Event #
 (most recent = 1)</t>
         </is>
       </c>
-      <c r="B56" s="30" t="inlineStr">
+      <c r="B56" s="31" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="C56" s="30" t="inlineStr">
+      <c r="C56" s="31" t="inlineStr">
         <is>
           <t>Time</t>
         </is>
       </c>
-      <c r="D56" s="30" t="inlineStr">
+      <c r="D56" s="31" t="inlineStr">
         <is>
           <t>Event Description / Type</t>
         </is>
       </c>
-      <c r="E56" s="26" t="n"/>
-    </row>
-    <row r="57" ht="15" customHeight="1" s="22">
-      <c r="A57" s="40" t="n">
+      <c r="E56" s="27" t="n"/>
+    </row>
+    <row r="57" ht="15" customHeight="1" s="23">
+      <c r="A57" s="41" t="n">
         <v>1</v>
       </c>
-      <c r="B57" s="28" t="n"/>
-      <c r="C57" s="28" t="n"/>
-      <c r="D57" s="28" t="n"/>
-      <c r="E57" s="26" t="n"/>
-    </row>
-    <row r="58" ht="15" customHeight="1" s="22">
-      <c r="A58" s="41" t="n">
+      <c r="B57" s="29" t="n"/>
+      <c r="C57" s="29" t="n"/>
+      <c r="D57" s="29" t="n"/>
+      <c r="E57" s="27" t="n"/>
+    </row>
+    <row r="58" ht="15" customHeight="1" s="23">
+      <c r="A58" s="42" t="n">
         <v>2</v>
       </c>
-      <c r="B58" s="38" t="n"/>
-      <c r="C58" s="38" t="n"/>
-      <c r="D58" s="38" t="n"/>
-      <c r="E58" s="26" t="n"/>
-    </row>
-    <row r="59" ht="15" customHeight="1" s="22">
-      <c r="A59" s="40" t="n">
+      <c r="B58" s="39" t="n"/>
+      <c r="C58" s="39" t="n"/>
+      <c r="D58" s="39" t="n"/>
+      <c r="E58" s="27" t="n"/>
+    </row>
+    <row r="59" ht="15" customHeight="1" s="23">
+      <c r="A59" s="41" t="n">
         <v>3</v>
       </c>
-      <c r="B59" s="28" t="n"/>
-      <c r="C59" s="28" t="n"/>
-      <c r="D59" s="28" t="n"/>
-      <c r="E59" s="26" t="n"/>
-    </row>
-    <row r="60" ht="15" customHeight="1" s="22">
-      <c r="A60" s="41" t="n">
+      <c r="B59" s="29" t="n"/>
+      <c r="C59" s="29" t="n"/>
+      <c r="D59" s="29" t="n"/>
+      <c r="E59" s="27" t="n"/>
+    </row>
+    <row r="60" ht="15" customHeight="1" s="23">
+      <c r="A60" s="42" t="n">
         <v>4</v>
       </c>
-      <c r="B60" s="38" t="n"/>
-      <c r="C60" s="38" t="n"/>
-      <c r="D60" s="38" t="n"/>
-      <c r="E60" s="26" t="n"/>
-    </row>
-    <row r="61" ht="15" customHeight="1" s="22">
-      <c r="A61" s="40" t="n">
+      <c r="B60" s="39" t="n"/>
+      <c r="C60" s="39" t="n"/>
+      <c r="D60" s="39" t="n"/>
+      <c r="E60" s="27" t="n"/>
+    </row>
+    <row r="61" ht="15" customHeight="1" s="23">
+      <c r="A61" s="41" t="n">
         <v>5</v>
       </c>
-      <c r="B61" s="28" t="n"/>
-      <c r="C61" s="28" t="n"/>
-      <c r="D61" s="28" t="n"/>
-      <c r="E61" s="26" t="n"/>
-    </row>
-    <row r="62" ht="15" customHeight="1" s="22">
-      <c r="A62" s="41" t="n">
+      <c r="B61" s="29" t="n"/>
+      <c r="C61" s="29" t="n"/>
+      <c r="D61" s="29" t="n"/>
+      <c r="E61" s="27" t="n"/>
+    </row>
+    <row r="62" ht="15" customHeight="1" s="23">
+      <c r="A62" s="42" t="n">
         <v>6</v>
       </c>
-      <c r="B62" s="38" t="n"/>
-      <c r="C62" s="38" t="n"/>
-      <c r="D62" s="38" t="n"/>
-      <c r="E62" s="26" t="n"/>
-    </row>
-    <row r="63" ht="15" customHeight="1" s="22">
-      <c r="A63" s="40" t="n">
+      <c r="B62" s="39" t="n"/>
+      <c r="C62" s="39" t="n"/>
+      <c r="D62" s="39" t="n"/>
+      <c r="E62" s="27" t="n"/>
+    </row>
+    <row r="63" ht="15" customHeight="1" s="23">
+      <c r="A63" s="41" t="n">
         <v>7</v>
       </c>
-      <c r="B63" s="28" t="n"/>
-      <c r="C63" s="28" t="n"/>
-      <c r="D63" s="28" t="n"/>
-      <c r="E63" s="26" t="n"/>
-    </row>
-    <row r="64" ht="15" customHeight="1" s="22">
-      <c r="A64" s="41" t="n">
+      <c r="B63" s="29" t="n"/>
+      <c r="C63" s="29" t="n"/>
+      <c r="D63" s="29" t="n"/>
+      <c r="E63" s="27" t="n"/>
+    </row>
+    <row r="64" ht="15" customHeight="1" s="23">
+      <c r="A64" s="42" t="n">
         <v>8</v>
       </c>
-      <c r="B64" s="38" t="n"/>
-      <c r="C64" s="38" t="n"/>
-      <c r="D64" s="38" t="n"/>
-      <c r="E64" s="26" t="n"/>
-    </row>
-    <row r="65" ht="15" customHeight="1" s="22">
-      <c r="A65" s="40" t="n">
+      <c r="B64" s="39" t="n"/>
+      <c r="C64" s="39" t="n"/>
+      <c r="D64" s="39" t="n"/>
+      <c r="E64" s="27" t="n"/>
+    </row>
+    <row r="65" ht="15" customHeight="1" s="23">
+      <c r="A65" s="41" t="n">
         <v>9</v>
       </c>
-      <c r="B65" s="28" t="n"/>
-      <c r="C65" s="28" t="n"/>
-      <c r="D65" s="28" t="n"/>
-      <c r="E65" s="26" t="n"/>
-    </row>
-    <row r="66" ht="15" customHeight="1" s="22">
-      <c r="A66" s="41" t="n">
+      <c r="B65" s="29" t="n"/>
+      <c r="C65" s="29" t="n"/>
+      <c r="D65" s="29" t="n"/>
+      <c r="E65" s="27" t="n"/>
+    </row>
+    <row r="66" ht="15" customHeight="1" s="23">
+      <c r="A66" s="42" t="n">
         <v>10</v>
       </c>
-      <c r="B66" s="38" t="n"/>
-      <c r="C66" s="38" t="n"/>
-      <c r="D66" s="38" t="n"/>
-      <c r="E66" s="26" t="n"/>
-    </row>
-    <row r="67" ht="15" customHeight="1" s="22">
-      <c r="A67" s="40" t="n">
+      <c r="B66" s="39" t="n"/>
+      <c r="C66" s="39" t="n"/>
+      <c r="D66" s="39" t="n"/>
+      <c r="E66" s="27" t="n"/>
+    </row>
+    <row r="67" ht="15" customHeight="1" s="23">
+      <c r="A67" s="41" t="n">
         <v>11</v>
       </c>
-      <c r="B67" s="28" t="n"/>
-      <c r="C67" s="28" t="n"/>
-      <c r="D67" s="28" t="n"/>
-      <c r="E67" s="26" t="n"/>
-    </row>
-    <row r="68" ht="15" customHeight="1" s="22">
-      <c r="A68" s="41" t="n">
+      <c r="B67" s="29" t="n"/>
+      <c r="C67" s="29" t="n"/>
+      <c r="D67" s="29" t="n"/>
+      <c r="E67" s="27" t="n"/>
+    </row>
+    <row r="68" ht="15" customHeight="1" s="23">
+      <c r="A68" s="42" t="n">
         <v>12</v>
       </c>
-      <c r="B68" s="38" t="n"/>
-      <c r="C68" s="38" t="n"/>
-      <c r="D68" s="38" t="n"/>
-      <c r="E68" s="26" t="n"/>
-    </row>
-    <row r="69" ht="15" customHeight="1" s="22">
-      <c r="A69" s="42" t="inlineStr">
+      <c r="B68" s="39" t="n"/>
+      <c r="C68" s="39" t="n"/>
+      <c r="D68" s="39" t="n"/>
+      <c r="E68" s="27" t="n"/>
+    </row>
+    <row r="69" ht="15" customHeight="1" s="23">
+      <c r="A69" s="43" t="inlineStr">
         <is>
           <t>Total events since last check (approx.)</t>
         </is>
       </c>
-      <c r="B69" s="28" t="n"/>
-      <c r="C69" s="25" t="n"/>
-      <c r="D69" s="25" t="n"/>
-      <c r="E69" s="26" t="n"/>
-    </row>
-    <row r="71" ht="18" customHeight="1" s="22">
-      <c r="A71" s="24" t="inlineStr">
+      <c r="B69" s="29" t="n"/>
+      <c r="C69" s="26" t="n"/>
+      <c r="D69" s="26" t="n"/>
+      <c r="E69" s="27" t="n"/>
+    </row>
+    <row r="71" ht="18" customHeight="1" s="23">
+      <c r="A71" s="25" t="inlineStr">
         <is>
           <t>7.  DCS / 800XA COMMUNICATION CHECK</t>
         </is>
       </c>
-      <c r="B71" s="25" t="n"/>
-      <c r="C71" s="25" t="n"/>
-      <c r="D71" s="25" t="n"/>
-      <c r="E71" s="26" t="n"/>
-    </row>
-    <row r="72" ht="36" customHeight="1" s="22">
-      <c r="A72" s="29" t="inlineStr">
+      <c r="B71" s="26" t="n"/>
+      <c r="C71" s="26" t="n"/>
+      <c r="D71" s="26" t="n"/>
+      <c r="E71" s="27" t="n"/>
+    </row>
+    <row r="72" ht="36" customHeight="1" s="23">
+      <c r="A72" s="30" t="inlineStr">
         <is>
           <t>Open the relay faceplate in ABB 800XA. Verify that live values (currents, status) are updating and not frozen. Check for any communication alarm objects (yellow/red). Record the 800XA object path or faceplate name below.</t>
         </is>
       </c>
-      <c r="B72" s="25" t="n"/>
-      <c r="C72" s="25" t="n"/>
-      <c r="D72" s="25" t="n"/>
-      <c r="E72" s="26" t="n"/>
-    </row>
-    <row r="73" ht="27.75" customHeight="1" s="22">
-      <c r="A73" s="30" t="inlineStr">
+      <c r="B72" s="26" t="n"/>
+      <c r="C72" s="26" t="n"/>
+      <c r="D72" s="26" t="n"/>
+      <c r="E72" s="27" t="n"/>
+    </row>
+    <row r="73" ht="27.75" customHeight="1" s="23">
+      <c r="A73" s="31" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
       </c>
-      <c r="B73" s="30" t="inlineStr">
+      <c r="B73" s="31" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="C73" s="30" t="inlineStr">
+      <c r="C73" s="31" t="inlineStr">
         <is>
           <t>Result
 (Y / N)</t>
         </is>
       </c>
-      <c r="D73" s="30" t="inlineStr">
+      <c r="D73" s="31" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="E73" s="26" t="n"/>
-    </row>
-    <row r="74" ht="15" customHeight="1" s="22">
-      <c r="A74" s="27" t="inlineStr">
+      <c r="E73" s="27" t="n"/>
+    </row>
+    <row r="74" ht="15" customHeight="1" s="23">
+      <c r="A74" s="28" t="inlineStr">
         <is>
           <t>800XA faceplate opened</t>
         </is>
       </c>
-      <c r="B74" s="35" t="inlineStr">
+      <c r="B74" s="36" t="inlineStr">
         <is>
           <t>Navigate to relay faceplate in 800XA control system</t>
         </is>
       </c>
-      <c r="C74" s="34" t="n"/>
-      <c r="D74" s="28" t="n"/>
-      <c r="E74" s="26" t="n"/>
-    </row>
-    <row r="75" ht="15" customHeight="1" s="22">
-      <c r="A75" s="27" t="inlineStr">
+      <c r="C74" s="35" t="n"/>
+      <c r="D74" s="29" t="n"/>
+      <c r="E74" s="27" t="n"/>
+    </row>
+    <row r="75" ht="15" customHeight="1" s="23">
+      <c r="A75" s="28" t="inlineStr">
         <is>
           <t>Live values updating</t>
         </is>
       </c>
-      <c r="B75" s="35" t="inlineStr">
+      <c r="B75" s="36" t="inlineStr">
         <is>
           <t>Phase currents / status visible and changing with load.</t>
         </is>
       </c>
-      <c r="C75" s="34" t="n"/>
-      <c r="D75" s="28" t="n"/>
-      <c r="E75" s="26" t="n"/>
-    </row>
-    <row r="76" ht="15" customHeight="1" s="22">
-      <c r="A76" s="27" t="inlineStr">
+      <c r="C75" s="35" t="n"/>
+      <c r="D75" s="29" t="n"/>
+      <c r="E75" s="27" t="n"/>
+    </row>
+    <row r="76" ht="15" customHeight="1" s="23">
+      <c r="A76" s="28" t="inlineStr">
         <is>
           <t>No communication alarm</t>
         </is>
       </c>
-      <c r="B76" s="35" t="inlineStr">
+      <c r="B76" s="36" t="inlineStr">
         <is>
           <t>No yellow or red communication alarm objects on faceplate</t>
         </is>
       </c>
-      <c r="C76" s="34" t="n"/>
-      <c r="D76" s="28" t="n"/>
-      <c r="E76" s="26" t="n"/>
-    </row>
-    <row r="77" ht="15" customHeight="1" s="22">
-      <c r="A77" s="42" t="inlineStr">
+      <c r="C76" s="35" t="n"/>
+      <c r="D76" s="29" t="n"/>
+      <c r="E76" s="27" t="n"/>
+    </row>
+    <row r="77" ht="15" customHeight="1" s="23">
+      <c r="A77" s="43" t="inlineStr">
         <is>
           <t>Record 800XA object path / faceplate name</t>
         </is>
       </c>
-      <c r="B77" s="35" t="inlineStr">
+      <c r="B77" s="36" t="inlineStr">
         <is>
           <t>e.g. "Site/Substation/Relay Tag/Faceplate"</t>
         </is>
       </c>
-      <c r="C77" s="34" t="n"/>
-      <c r="D77" s="28" t="n"/>
-      <c r="E77" s="26" t="n"/>
-    </row>
-    <row r="79" ht="18" customHeight="1" s="22">
-      <c r="A79" s="24" t="inlineStr">
+      <c r="C77" s="35" t="n"/>
+      <c r="D77" s="29" t="n"/>
+      <c r="E77" s="27" t="n"/>
+    </row>
+    <row r="79" ht="18" customHeight="1" s="23">
+      <c r="A79" s="25" t="inlineStr">
         <is>
           <t>8.  OPTIONAL — CLEAR EVENT BUFFERS  (only if required by your procedure)</t>
         </is>
       </c>
-      <c r="B79" s="25" t="n"/>
-      <c r="C79" s="25" t="n"/>
-      <c r="D79" s="25" t="n"/>
-      <c r="E79" s="26" t="n"/>
-    </row>
-    <row r="80" ht="31.5" customHeight="1" s="22">
-      <c r="A80" s="43" t="inlineStr">
+      <c r="B79" s="26" t="n"/>
+      <c r="C79" s="26" t="n"/>
+      <c r="D79" s="26" t="n"/>
+      <c r="E79" s="27" t="n"/>
+    </row>
+    <row r="80" ht="31.5" customHeight="1" s="23">
+      <c r="A80" s="44" t="inlineStr">
         <is>
           <t>If your site procedure requires clearing event buffers after recording, issue the following serial commands at Access Level 1 or 2. Ensure all events have been downloaded/recorded BEFORE clearing.</t>
         </is>
       </c>
-      <c r="B80" s="25" t="n"/>
-      <c r="C80" s="25" t="n"/>
-      <c r="D80" s="25" t="n"/>
-      <c r="E80" s="26" t="n"/>
-    </row>
-    <row r="81" ht="27.75" customHeight="1" s="22">
-      <c r="A81" s="30" t="inlineStr">
+      <c r="B80" s="26" t="n"/>
+      <c r="C80" s="26" t="n"/>
+      <c r="D80" s="26" t="n"/>
+      <c r="E80" s="27" t="n"/>
+    </row>
+    <row r="81" ht="27.75" customHeight="1" s="23">
+      <c r="A81" s="31" t="inlineStr">
         <is>
           <t>Serial Command</t>
         </is>
       </c>
-      <c r="B81" s="30" t="inlineStr">
+      <c r="B81" s="31" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="C81" s="30" t="inlineStr">
+      <c r="C81" s="31" t="inlineStr">
         <is>
           <t>Performed?
 (Y / N / N/A)</t>
         </is>
       </c>
-      <c r="D81" s="30" t="inlineStr">
+      <c r="D81" s="31" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="E81" s="26" t="n"/>
-    </row>
-    <row r="82" ht="15" customHeight="1" s="22">
-      <c r="A82" s="27" t="inlineStr">
+      <c r="E81" s="27" t="n"/>
+    </row>
+    <row r="82" ht="15" customHeight="1" s="23">
+      <c r="A82" s="28" t="inlineStr">
         <is>
           <t>SUM R &lt;Enter&gt;</t>
         </is>
       </c>
-      <c r="B82" s="35" t="inlineStr">
+      <c r="B82" s="36" t="inlineStr">
         <is>
           <t>Reset event report and Summary Command buffers</t>
         </is>
       </c>
-      <c r="C82" s="34" t="n"/>
-      <c r="D82" s="28" t="n"/>
-      <c r="E82" s="26" t="n"/>
-    </row>
-    <row r="83" ht="15" customHeight="1" s="22">
-      <c r="A83" s="27" t="inlineStr">
+      <c r="C82" s="35" t="n"/>
+      <c r="D82" s="29" t="n"/>
+      <c r="E82" s="27" t="n"/>
+    </row>
+    <row r="83" ht="15" customHeight="1" s="23">
+      <c r="A83" s="28" t="inlineStr">
         <is>
           <t>SER R &lt;Enter&gt;</t>
         </is>
       </c>
-      <c r="B83" s="35" t="inlineStr">
+      <c r="B83" s="36" t="inlineStr">
         <is>
           <t>Reset Sequential Events Record buffer</t>
         </is>
       </c>
-      <c r="C83" s="34" t="n"/>
-      <c r="D83" s="28" t="n"/>
-      <c r="E83" s="26" t="n"/>
-    </row>
-    <row r="84" ht="15" customHeight="1" s="22">
-      <c r="A84" s="27" t="inlineStr">
+      <c r="C83" s="35" t="n"/>
+      <c r="D83" s="29" t="n"/>
+      <c r="E83" s="27" t="n"/>
+    </row>
+    <row r="84" ht="15" customHeight="1" s="23">
+      <c r="A84" s="28" t="inlineStr">
         <is>
           <t>HIS C &lt;Enter&gt;</t>
         </is>
       </c>
-      <c r="B84" s="35" t="inlineStr">
+      <c r="B84" s="36" t="inlineStr">
         <is>
           <t>Clear event history (if required — confirm with supervisor)</t>
         </is>
       </c>
-      <c r="C84" s="34" t="n"/>
-      <c r="D84" s="28" t="n"/>
-      <c r="E84" s="26" t="n"/>
-    </row>
-    <row r="86" ht="18" customHeight="1" s="22">
-      <c r="A86" s="24" t="inlineStr">
+      <c r="C84" s="35" t="n"/>
+      <c r="D84" s="29" t="n"/>
+      <c r="E84" s="27" t="n"/>
+    </row>
+    <row r="86" ht="18" customHeight="1" s="23">
+      <c r="A86" s="25" t="inlineStr">
         <is>
           <t>9.  OBSERVATIONS AND CORRECTIVE ACTIONS</t>
         </is>
       </c>
-      <c r="B86" s="25" t="n"/>
-      <c r="C86" s="25" t="n"/>
-      <c r="D86" s="25" t="n"/>
-      <c r="E86" s="26" t="n"/>
-    </row>
-    <row r="87" ht="18" customHeight="1" s="22">
-      <c r="A87" s="44" t="n"/>
-      <c r="B87" s="45" t="n"/>
-      <c r="C87" s="45" t="n"/>
-      <c r="D87" s="45" t="n"/>
-      <c r="E87" s="46" t="n"/>
-    </row>
-    <row r="88" ht="18" customHeight="1" s="22">
-      <c r="A88" s="47" t="n"/>
-      <c r="E88" s="48" t="n"/>
-    </row>
-    <row r="89" ht="18" customHeight="1" s="22">
-      <c r="A89" s="47" t="n"/>
-      <c r="E89" s="48" t="n"/>
-    </row>
-    <row r="90" ht="18" customHeight="1" s="22">
-      <c r="A90" s="47" t="n"/>
-      <c r="E90" s="48" t="n"/>
-    </row>
-    <row r="91" ht="18" customHeight="1" s="22">
-      <c r="A91" s="49" t="n"/>
-      <c r="B91" s="50" t="n"/>
-      <c r="C91" s="50" t="n"/>
-      <c r="D91" s="50" t="n"/>
-      <c r="E91" s="51" t="n"/>
-    </row>
-    <row r="93" ht="18" customHeight="1" s="22">
-      <c r="A93" s="24" t="inlineStr">
+      <c r="B86" s="26" t="n"/>
+      <c r="C86" s="26" t="n"/>
+      <c r="D86" s="26" t="n"/>
+      <c r="E86" s="27" t="n"/>
+    </row>
+    <row r="87" ht="18" customHeight="1" s="23">
+      <c r="A87" s="45" t="n"/>
+      <c r="B87" s="46" t="n"/>
+      <c r="C87" s="46" t="n"/>
+      <c r="D87" s="46" t="n"/>
+      <c r="E87" s="47" t="n"/>
+    </row>
+    <row r="88" ht="18" customHeight="1" s="23">
+      <c r="A88" s="48" t="n"/>
+      <c r="E88" s="49" t="n"/>
+    </row>
+    <row r="89" ht="18" customHeight="1" s="23">
+      <c r="A89" s="48" t="n"/>
+      <c r="E89" s="49" t="n"/>
+    </row>
+    <row r="90" ht="18" customHeight="1" s="23">
+      <c r="A90" s="48" t="n"/>
+      <c r="E90" s="49" t="n"/>
+    </row>
+    <row r="91" ht="18" customHeight="1" s="23">
+      <c r="A91" s="50" t="n"/>
+      <c r="B91" s="51" t="n"/>
+      <c r="C91" s="51" t="n"/>
+      <c r="D91" s="51" t="n"/>
+      <c r="E91" s="52" t="n"/>
+    </row>
+    <row r="93" ht="18" customHeight="1" s="23">
+      <c r="A93" s="25" t="inlineStr">
         <is>
           <t>10.  SIGN-OFF</t>
         </is>
       </c>
-      <c r="B93" s="25" t="n"/>
-      <c r="C93" s="25" t="n"/>
-      <c r="D93" s="25" t="n"/>
-      <c r="E93" s="26" t="n"/>
-    </row>
-    <row r="94" ht="27.75" customHeight="1" s="22">
-      <c r="A94" s="30" t="inlineStr">
+      <c r="B93" s="26" t="n"/>
+      <c r="C93" s="26" t="n"/>
+      <c r="D93" s="26" t="n"/>
+      <c r="E93" s="27" t="n"/>
+    </row>
+    <row r="94" ht="27.75" customHeight="1" s="23">
+      <c r="A94" s="31" t="inlineStr">
         <is>
           <t>Role</t>
         </is>
       </c>
-      <c r="B94" s="30" t="inlineStr">
+      <c r="B94" s="31" t="inlineStr">
         <is>
           <t>Name (print)</t>
         </is>
       </c>
-      <c r="C94" s="30" t="inlineStr">
+      <c r="C94" s="31" t="inlineStr">
         <is>
           <t>Signature</t>
         </is>
       </c>
-      <c r="D94" s="30" t="inlineStr">
+      <c r="D94" s="31" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="E94" s="26" t="n"/>
-    </row>
-    <row r="95" ht="24" customHeight="1" s="22">
-      <c r="A95" s="27" t="inlineStr">
+      <c r="E94" s="27" t="n"/>
+    </row>
+    <row r="95" ht="24" customHeight="1" s="23">
+      <c r="A95" s="28" t="inlineStr">
         <is>
           <t>Technician</t>
         </is>
       </c>
-      <c r="B95" s="28" t="n"/>
-      <c r="C95" s="28" t="n"/>
-      <c r="D95" s="28" t="n"/>
-      <c r="E95" s="26" t="n"/>
-    </row>
-    <row r="96" ht="24" customHeight="1" s="22">
-      <c r="A96" s="27" t="inlineStr">
+      <c r="B95" s="29" t="n"/>
+      <c r="C95" s="29" t="n"/>
+      <c r="D95" s="29" t="n"/>
+      <c r="E95" s="27" t="n"/>
+    </row>
+    <row r="96" ht="24" customHeight="1" s="23">
+      <c r="A96" s="28" t="inlineStr">
         <is>
           <t>Supervisor / Witness</t>
         </is>
       </c>
-      <c r="B96" s="28" t="n"/>
-      <c r="C96" s="28" t="n"/>
-      <c r="D96" s="28" t="n"/>
-      <c r="E96" s="26" t="n"/>
+      <c r="B96" s="29" t="n"/>
+      <c r="C96" s="29" t="n"/>
+      <c r="D96" s="29" t="n"/>
+      <c r="E96" s="27" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="54">
@@ -1929,7 +1932,7 @@
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentOddEven="0" differentFirst="0">
     <oddHeader/>
-    <oddFooter>&amp;L&amp;"Calibri,Bold"&amp;8 &amp;K1F4E79&amp;BContact Energy&amp;C&amp;8 SEL Biennial Visual Check&amp;R&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;"Calibri,Bold"&amp;8 &amp;"Calibri,Regular"&amp;8 &amp;K1F4E79&amp;BContact Energy&amp;C&amp;8 SEL Biennial Visual Check&amp;R&amp;8 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter>&amp;L&amp;8 &amp;K1F4E79&amp;BContact Energy&amp;C&amp;8 SEL Biennial Visual Check&amp;R&amp;8 Page &amp;P of &amp;N</evenFooter>
     <firstHeader/>

</xml_diff>